<commit_message>
Q1 2026 SNA Update
</commit_message>
<xml_diff>
--- a/Data/National Accounts/PSA-02HFCE_2018PSNA_Qrt.xlsx
+++ b/Data/National Accounts/PSA-02HFCE_2018PSNA_Qrt.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\Shared drives\QNAP\NAP Dissemination\As of April 2026\Tables\NAP Q1 2000 to Q4 2025\Qtr\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Shared drives\QNAP\NAP Dissemination\As of May 2026\Tables\NAP Q1 2000 to Q1 2026\Qtr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{109C37CB-0206-4D93-9F2F-F0CD23AD5279}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E40A17C-6613-41F7-A73A-5E7AE0B57C73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="794" xr2:uid="{736930C2-BFBB-46C3-AE9E-AECFC8C3145D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="794" xr2:uid="{736930C2-BFBB-46C3-AE9E-AECFC8C3145D}"/>
   </bookViews>
   <sheets>
     <sheet name="HFCE" sheetId="2" r:id="rId1"/>
@@ -521,7 +521,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="916" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="64">
   <si>
     <t>National Accounts of the Philippines</t>
   </si>
@@ -707,10 +707,13 @@
     <t>Percent Share, at Constant 2018 Prices</t>
   </si>
   <si>
-    <t>Q1 2000 to Q4 2025</t>
+    <t>Q1 2000 to Q1 2026</t>
   </si>
   <si>
-    <t>As of April 2026</t>
+    <t>As of May 2026</t>
+  </si>
+  <si>
+    <t>2025 - 2026</t>
   </si>
 </sst>
 </file>
@@ -1244,8 +1247,8 @@
     <col min="75" max="77" width="16.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="78" max="78" width="16.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="79" max="93" width="16.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="94" max="105" width="16.42578125" style="22" bestFit="1" customWidth="1"/>
-    <col min="106" max="16384" width="10" style="1"/>
+    <col min="94" max="106" width="16.42578125" style="22" bestFit="1" customWidth="1"/>
+    <col min="107" max="16384" width="10" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:179" x14ac:dyDescent="0.2">
@@ -1436,6 +1439,9 @@
       <c r="CY9" s="23"/>
       <c r="CZ9" s="23"/>
       <c r="DA9" s="23"/>
+      <c r="DB9" s="23">
+        <v>2026</v>
+      </c>
     </row>
     <row r="10" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
@@ -1752,6 +1758,9 @@
       </c>
       <c r="DA10" s="24" t="s">
         <v>5</v>
+      </c>
+      <c r="DB10" s="24" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:179" ht="10.9" customHeight="1" x14ac:dyDescent="0.2">
@@ -2073,7 +2082,9 @@
       <c r="DA12" s="25">
         <v>2257594.2514206418</v>
       </c>
-      <c r="DB12" s="8"/>
+      <c r="DB12" s="25">
+        <v>1778620.7258560532</v>
+      </c>
       <c r="DC12" s="8"/>
       <c r="DD12" s="8"/>
       <c r="DE12" s="8"/>
@@ -2464,7 +2475,9 @@
       <c r="DA13" s="25">
         <v>120252.82278633314</v>
       </c>
-      <c r="DB13" s="8"/>
+      <c r="DB13" s="25">
+        <v>98345.741683448505</v>
+      </c>
       <c r="DC13" s="8"/>
       <c r="DD13" s="8"/>
       <c r="DE13" s="8"/>
@@ -2855,7 +2868,9 @@
       <c r="DA14" s="25">
         <v>94741.452218738676</v>
       </c>
-      <c r="DB14" s="8"/>
+      <c r="DB14" s="25">
+        <v>75003.247061091388</v>
+      </c>
       <c r="DC14" s="8"/>
       <c r="DD14" s="8"/>
       <c r="DE14" s="8"/>
@@ -3246,7 +3261,9 @@
       <c r="DA15" s="25">
         <v>631565.8971390489</v>
       </c>
-      <c r="DB15" s="8"/>
+      <c r="DB15" s="25">
+        <v>597623.12105468463</v>
+      </c>
       <c r="DC15" s="8"/>
       <c r="DD15" s="8"/>
       <c r="DE15" s="8"/>
@@ -3637,7 +3654,9 @@
       <c r="DA16" s="25">
         <v>147486.66570831661</v>
       </c>
-      <c r="DB16" s="8"/>
+      <c r="DB16" s="25">
+        <v>129497.11240136674</v>
+      </c>
       <c r="DC16" s="8"/>
       <c r="DD16" s="8"/>
       <c r="DE16" s="8"/>
@@ -4028,7 +4047,9 @@
       <c r="DA17" s="25">
         <v>269475.82895237411</v>
       </c>
-      <c r="DB17" s="8"/>
+      <c r="DB17" s="25">
+        <v>250472.03487425239</v>
+      </c>
       <c r="DC17" s="8"/>
       <c r="DD17" s="8"/>
       <c r="DE17" s="8"/>
@@ -4419,7 +4440,9 @@
       <c r="DA18" s="25">
         <v>496667.21270987199</v>
       </c>
-      <c r="DB18" s="8"/>
+      <c r="DB18" s="25">
+        <v>595479.16807577095</v>
+      </c>
       <c r="DC18" s="8"/>
       <c r="DD18" s="8"/>
       <c r="DE18" s="8"/>
@@ -4810,7 +4833,9 @@
       <c r="DA19" s="25">
         <v>145667.37342405706</v>
       </c>
-      <c r="DB19" s="8"/>
+      <c r="DB19" s="25">
+        <v>151721.68295889723</v>
+      </c>
       <c r="DC19" s="8"/>
       <c r="DD19" s="8"/>
       <c r="DE19" s="8"/>
@@ -5201,7 +5226,9 @@
       <c r="DA20" s="25">
         <v>116085.0135024778</v>
       </c>
-      <c r="DB20" s="8"/>
+      <c r="DB20" s="25">
+        <v>104579.21517266936</v>
+      </c>
       <c r="DC20" s="8"/>
       <c r="DD20" s="8"/>
       <c r="DE20" s="8"/>
@@ -5592,7 +5619,9 @@
       <c r="DA21" s="25">
         <v>300009.49537248426</v>
       </c>
-      <c r="DB21" s="8"/>
+      <c r="DB21" s="25">
+        <v>301333.79849671648</v>
+      </c>
       <c r="DC21" s="8"/>
       <c r="DD21" s="8"/>
       <c r="DE21" s="8"/>
@@ -5983,7 +6012,9 @@
       <c r="DA22" s="25">
         <v>550139.20937379065</v>
       </c>
-      <c r="DB22" s="8"/>
+      <c r="DB22" s="25">
+        <v>591401.75434679841</v>
+      </c>
       <c r="DC22" s="8"/>
       <c r="DD22" s="8"/>
       <c r="DE22" s="8"/>
@@ -6374,7 +6405,9 @@
       <c r="DA23" s="25">
         <v>913942.70429242158</v>
       </c>
-      <c r="DB23" s="8"/>
+      <c r="DB23" s="25">
+        <v>778827.55687577662</v>
+      </c>
       <c r="DC23" s="8"/>
       <c r="DD23" s="8"/>
       <c r="DE23" s="8"/>
@@ -6554,7 +6587,7 @@
       <c r="CY24" s="26"/>
       <c r="CZ24" s="26"/>
       <c r="DA24" s="26"/>
-      <c r="DB24" s="8"/>
+      <c r="DB24" s="26"/>
       <c r="DC24" s="8"/>
       <c r="DD24" s="8"/>
       <c r="DE24" s="8"/>
@@ -6945,7 +6978,9 @@
       <c r="DA25" s="10">
         <v>6043627.9269005563</v>
       </c>
-      <c r="DB25" s="8"/>
+      <c r="DB25" s="10">
+        <v>5452905.1588575263</v>
+      </c>
       <c r="DC25" s="8"/>
       <c r="DD25" s="8"/>
       <c r="DE25" s="8"/>
@@ -7126,6 +7161,7 @@
       <c r="CY26" s="27"/>
       <c r="CZ26" s="27"/>
       <c r="DA26" s="27"/>
+      <c r="DB26" s="27"/>
     </row>
     <row r="27" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A27" s="12" t="s">
@@ -7237,7 +7273,7 @@
       <c r="CY28" s="15"/>
       <c r="CZ28" s="15"/>
       <c r="DA28" s="15"/>
-      <c r="DB28" s="8"/>
+      <c r="DB28" s="15"/>
       <c r="DC28" s="8"/>
       <c r="DD28" s="8"/>
       <c r="DE28" s="8"/>
@@ -7417,7 +7453,7 @@
       <c r="CY29" s="17"/>
       <c r="CZ29" s="17"/>
       <c r="DA29" s="17"/>
-      <c r="DB29" s="8"/>
+      <c r="DB29" s="17"/>
       <c r="DC29" s="8"/>
       <c r="DD29" s="8"/>
       <c r="DE29" s="8"/>
@@ -7680,6 +7716,9 @@
       <c r="CY38" s="23"/>
       <c r="CZ38" s="23"/>
       <c r="DA38" s="23"/>
+      <c r="DB38" s="23">
+        <v>2026</v>
+      </c>
     </row>
     <row r="39" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
@@ -7996,6 +8035,9 @@
       </c>
       <c r="DA39" s="24" t="s">
         <v>5</v>
+      </c>
+      <c r="DB39" s="24" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:179" ht="10.9" customHeight="1" x14ac:dyDescent="0.2">
@@ -8317,7 +8359,9 @@
       <c r="DA41" s="25">
         <v>1712013.4937564556</v>
       </c>
-      <c r="DB41" s="18"/>
+      <c r="DB41" s="25">
+        <v>1336154.8218690488</v>
+      </c>
       <c r="DC41" s="18"/>
       <c r="DD41" s="18"/>
       <c r="DE41" s="8"/>
@@ -8708,7 +8752,9 @@
       <c r="DA42" s="25">
         <v>66940.263586569476</v>
       </c>
-      <c r="DB42" s="18"/>
+      <c r="DB42" s="25">
+        <v>54688.87528240637</v>
+      </c>
       <c r="DC42" s="18"/>
       <c r="DD42" s="18"/>
       <c r="DE42" s="8"/>
@@ -9099,7 +9145,9 @@
       <c r="DA43" s="25">
         <v>80447.531696095204</v>
       </c>
-      <c r="DB43" s="18"/>
+      <c r="DB43" s="25">
+        <v>62434.382449917008</v>
+      </c>
       <c r="DC43" s="18"/>
       <c r="DD43" s="18"/>
       <c r="DE43" s="8"/>
@@ -9490,7 +9538,9 @@
       <c r="DA44" s="25">
         <v>501771.40644787182</v>
       </c>
-      <c r="DB44" s="18"/>
+      <c r="DB44" s="25">
+        <v>497262.88891400094</v>
+      </c>
       <c r="DC44" s="18"/>
       <c r="DD44" s="18"/>
       <c r="DE44" s="8"/>
@@ -9881,7 +9931,9 @@
       <c r="DA45" s="25">
         <v>120110.55217656854</v>
       </c>
-      <c r="DB45" s="18"/>
+      <c r="DB45" s="25">
+        <v>100491.98654809655</v>
+      </c>
       <c r="DC45" s="18"/>
       <c r="DD45" s="18"/>
       <c r="DE45" s="8"/>
@@ -10272,7 +10324,9 @@
       <c r="DA46" s="25">
         <v>215584.36277543131</v>
       </c>
-      <c r="DB46" s="18"/>
+      <c r="DB46" s="25">
+        <v>204006.31705912558</v>
+      </c>
       <c r="DC46" s="18"/>
       <c r="DD46" s="18"/>
       <c r="DE46" s="8"/>
@@ -10663,7 +10717,9 @@
       <c r="DA47" s="25">
         <v>391363.50081725052</v>
       </c>
-      <c r="DB47" s="18"/>
+      <c r="DB47" s="25">
+        <v>432120.48511203448</v>
+      </c>
       <c r="DC47" s="18"/>
       <c r="DD47" s="18"/>
       <c r="DE47" s="8"/>
@@ -11054,7 +11110,9 @@
       <c r="DA48" s="25">
         <v>146789.74867700256</v>
       </c>
-      <c r="DB48" s="18"/>
+      <c r="DB48" s="25">
+        <v>141552.55683161606</v>
+      </c>
       <c r="DC48" s="18"/>
       <c r="DD48" s="18"/>
       <c r="DE48" s="8"/>
@@ -11445,7 +11503,9 @@
       <c r="DA49" s="25">
         <v>98793.237167360829</v>
       </c>
-      <c r="DB49" s="18"/>
+      <c r="DB49" s="25">
+        <v>86892.299465529941</v>
+      </c>
       <c r="DC49" s="18"/>
       <c r="DD49" s="18"/>
       <c r="DE49" s="8"/>
@@ -11836,7 +11896,9 @@
       <c r="DA50" s="25">
         <v>262734.49458966724</v>
       </c>
-      <c r="DB50" s="18"/>
+      <c r="DB50" s="25">
+        <v>250320.96917270299</v>
+      </c>
       <c r="DC50" s="18"/>
       <c r="DD50" s="18"/>
       <c r="DE50" s="8"/>
@@ -12227,7 +12289,9 @@
       <c r="DA51" s="25">
         <v>420188.94427363185</v>
       </c>
-      <c r="DB51" s="18"/>
+      <c r="DB51" s="25">
+        <v>435387.79461113992</v>
+      </c>
       <c r="DC51" s="18"/>
       <c r="DD51" s="18"/>
       <c r="DE51" s="8"/>
@@ -12618,7 +12682,9 @@
       <c r="DA52" s="25">
         <v>789234.57327706018</v>
       </c>
-      <c r="DB52" s="18"/>
+      <c r="DB52" s="25">
+        <v>591202.12934509362</v>
+      </c>
       <c r="DC52" s="18"/>
       <c r="DD52" s="18"/>
       <c r="DE52" s="8"/>
@@ -12798,7 +12864,7 @@
       <c r="CY53" s="26"/>
       <c r="CZ53" s="26"/>
       <c r="DA53" s="26"/>
-      <c r="DB53" s="8"/>
+      <c r="DB53" s="26"/>
       <c r="DC53" s="8"/>
       <c r="DD53" s="8"/>
       <c r="DE53" s="8"/>
@@ -13189,7 +13255,9 @@
       <c r="DA54" s="10">
         <v>4805972.1092409659</v>
       </c>
-      <c r="DB54" s="8"/>
+      <c r="DB54" s="10">
+        <v>4192515.5066607129</v>
+      </c>
       <c r="DC54" s="8"/>
       <c r="DD54" s="8"/>
       <c r="DE54" s="8"/>
@@ -13370,6 +13438,7 @@
       <c r="CY55" s="27"/>
       <c r="CZ55" s="27"/>
       <c r="DA55" s="27"/>
+      <c r="DB55" s="27"/>
     </row>
     <row r="56" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A56" s="12" t="s">
@@ -13481,7 +13550,7 @@
       <c r="CY57" s="26"/>
       <c r="CZ57" s="26"/>
       <c r="DA57" s="26"/>
-      <c r="DB57" s="8"/>
+      <c r="DB57" s="26"/>
       <c r="DC57" s="8"/>
       <c r="DD57" s="8"/>
       <c r="DE57" s="8"/>
@@ -13661,7 +13730,7 @@
       <c r="CY58" s="17"/>
       <c r="CZ58" s="17"/>
       <c r="DA58" s="17"/>
-      <c r="DB58" s="8"/>
+      <c r="DB58" s="17"/>
       <c r="DC58" s="8"/>
       <c r="DD58" s="8"/>
       <c r="DE58" s="8"/>
@@ -13757,6 +13826,7 @@
       <c r="CY61" s="28"/>
       <c r="CZ61" s="28"/>
       <c r="DA61" s="28"/>
+      <c r="DB61" s="28"/>
     </row>
     <row r="62" spans="1:179" x14ac:dyDescent="0.2">
       <c r="CT62" s="28"/>
@@ -13766,6 +13836,7 @@
       <c r="CY62" s="28"/>
       <c r="CZ62" s="28"/>
       <c r="DA62" s="28"/>
+      <c r="DB62" s="28"/>
     </row>
     <row r="63" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
@@ -13778,6 +13849,7 @@
       <c r="CY63" s="28"/>
       <c r="CZ63" s="28"/>
       <c r="DA63" s="28"/>
+      <c r="DB63" s="28"/>
     </row>
     <row r="64" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
@@ -13787,6 +13859,7 @@
       <c r="CY64" s="28"/>
       <c r="CZ64" s="28"/>
       <c r="DA64" s="28"/>
+      <c r="DB64" s="28"/>
     </row>
     <row r="65" spans="1:175" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
@@ -13796,12 +13869,13 @@
       <c r="CY65" s="29"/>
       <c r="CZ65" s="29"/>
       <c r="DA65" s="29"/>
+      <c r="DB65" s="29"/>
     </row>
     <row r="66" spans="1:175" x14ac:dyDescent="0.2">
-      <c r="CX66" s="29"/>
       <c r="CY66" s="29"/>
       <c r="CZ66" s="29"/>
       <c r="DA66" s="29"/>
+      <c r="DB66" s="29"/>
     </row>
     <row r="67" spans="1:175" x14ac:dyDescent="0.2">
       <c r="A67" s="3"/>
@@ -13955,10 +14029,13 @@
       <c r="CU67" s="23"/>
       <c r="CV67" s="23"/>
       <c r="CW67" s="23"/>
-      <c r="CX67" s="30"/>
+      <c r="CX67" s="23" t="s">
+        <v>63</v>
+      </c>
       <c r="CY67" s="30"/>
       <c r="CZ67" s="30"/>
       <c r="DA67" s="30"/>
+      <c r="DB67" s="30"/>
     </row>
     <row r="68" spans="1:175" x14ac:dyDescent="0.2">
       <c r="A68" s="4" t="s">
@@ -14264,17 +14341,20 @@
       <c r="CW68" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="CX68" s="31"/>
+      <c r="CX68" s="24" t="s">
+        <v>2</v>
+      </c>
       <c r="CY68" s="31"/>
       <c r="CZ68" s="31"/>
       <c r="DA68" s="31"/>
+      <c r="DB68" s="31"/>
     </row>
     <row r="69" spans="1:175" ht="10.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="6"/>
-      <c r="CX69" s="29"/>
       <c r="CY69" s="29"/>
       <c r="CZ69" s="29"/>
       <c r="DA69" s="29"/>
+      <c r="DB69" s="29"/>
     </row>
     <row r="70" spans="1:175" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
@@ -14580,11 +14660,13 @@
       <c r="CW70" s="32">
         <v>4.5040021672833319</v>
       </c>
-      <c r="CX70" s="33"/>
+      <c r="CX70" s="32">
+        <v>2.2521765703352798</v>
+      </c>
       <c r="CY70" s="33"/>
       <c r="CZ70" s="33"/>
       <c r="DA70" s="33"/>
-      <c r="DB70" s="8"/>
+      <c r="DB70" s="33"/>
       <c r="DC70" s="8"/>
       <c r="DD70" s="8"/>
       <c r="DE70" s="8"/>
@@ -14959,11 +15041,13 @@
       <c r="CW71" s="32">
         <v>-2.6867580532877611</v>
       </c>
-      <c r="CX71" s="33"/>
+      <c r="CX71" s="32">
+        <v>6.4741941354012198</v>
+      </c>
       <c r="CY71" s="33"/>
       <c r="CZ71" s="33"/>
       <c r="DA71" s="33"/>
-      <c r="DB71" s="8"/>
+      <c r="DB71" s="33"/>
       <c r="DC71" s="8"/>
       <c r="DD71" s="8"/>
       <c r="DE71" s="8"/>
@@ -15338,11 +15422,13 @@
       <c r="CW72" s="32">
         <v>0.85425742935640869</v>
       </c>
-      <c r="CX72" s="33"/>
+      <c r="CX72" s="32">
+        <v>15.005754421105095</v>
+      </c>
       <c r="CY72" s="33"/>
       <c r="CZ72" s="33"/>
       <c r="DA72" s="33"/>
-      <c r="DB72" s="8"/>
+      <c r="DB72" s="33"/>
       <c r="DC72" s="8"/>
       <c r="DD72" s="8"/>
       <c r="DE72" s="8"/>
@@ -15717,11 +15803,13 @@
       <c r="CW73" s="32">
         <v>2.8177282016049929</v>
       </c>
-      <c r="CX73" s="33"/>
+      <c r="CX73" s="32">
+        <v>6.6055781133850644</v>
+      </c>
       <c r="CY73" s="33"/>
       <c r="CZ73" s="33"/>
       <c r="DA73" s="33"/>
-      <c r="DB73" s="8"/>
+      <c r="DB73" s="33"/>
       <c r="DC73" s="8"/>
       <c r="DD73" s="8"/>
       <c r="DE73" s="8"/>
@@ -16096,11 +16184,13 @@
       <c r="CW74" s="32">
         <v>6.2002573040501829E-2</v>
       </c>
-      <c r="CX74" s="33"/>
+      <c r="CX74" s="32">
+        <v>5.9292585985969453</v>
+      </c>
       <c r="CY74" s="33"/>
       <c r="CZ74" s="33"/>
       <c r="DA74" s="33"/>
-      <c r="DB74" s="8"/>
+      <c r="DB74" s="33"/>
       <c r="DC74" s="8"/>
       <c r="DD74" s="8"/>
       <c r="DE74" s="8"/>
@@ -16475,11 +16565,13 @@
       <c r="CW75" s="32">
         <v>8.517487380089122</v>
       </c>
-      <c r="CX75" s="33"/>
+      <c r="CX75" s="32">
+        <v>9.0823825021554256</v>
+      </c>
       <c r="CY75" s="33"/>
       <c r="CZ75" s="33"/>
       <c r="DA75" s="33"/>
-      <c r="DB75" s="8"/>
+      <c r="DB75" s="33"/>
       <c r="DC75" s="8"/>
       <c r="DD75" s="8"/>
       <c r="DE75" s="8"/>
@@ -16854,11 +16946,13 @@
       <c r="CW76" s="32">
         <v>7.0480931519140881</v>
       </c>
-      <c r="CX76" s="33"/>
+      <c r="CX76" s="32">
+        <v>6.748168166432734</v>
+      </c>
       <c r="CY76" s="33"/>
       <c r="CZ76" s="33"/>
       <c r="DA76" s="33"/>
-      <c r="DB76" s="8"/>
+      <c r="DB76" s="33"/>
       <c r="DC76" s="8"/>
       <c r="DD76" s="8"/>
       <c r="DE76" s="8"/>
@@ -17233,11 +17327,13 @@
       <c r="CW77" s="32">
         <v>4.245173815947993</v>
       </c>
-      <c r="CX77" s="33"/>
+      <c r="CX77" s="32">
+        <v>6.4283724753448723</v>
+      </c>
       <c r="CY77" s="33"/>
       <c r="CZ77" s="33"/>
       <c r="DA77" s="33"/>
-      <c r="DB77" s="8"/>
+      <c r="DB77" s="33"/>
       <c r="DC77" s="8"/>
       <c r="DD77" s="8"/>
       <c r="DE77" s="8"/>
@@ -17612,11 +17708,13 @@
       <c r="CW78" s="32">
         <v>9.0856460685615872</v>
       </c>
-      <c r="CX78" s="33"/>
+      <c r="CX78" s="32">
+        <v>9.4690483265493128</v>
+      </c>
       <c r="CY78" s="33"/>
       <c r="CZ78" s="33"/>
       <c r="DA78" s="33"/>
-      <c r="DB78" s="8"/>
+      <c r="DB78" s="33"/>
       <c r="DC78" s="8"/>
       <c r="DD78" s="8"/>
       <c r="DE78" s="8"/>
@@ -17991,11 +18089,13 @@
       <c r="CW79" s="32">
         <v>9.8287101496879643</v>
       </c>
-      <c r="CX79" s="33"/>
+      <c r="CX79" s="32">
+        <v>9.8047587741586</v>
+      </c>
       <c r="CY79" s="33"/>
       <c r="CZ79" s="33"/>
       <c r="DA79" s="33"/>
-      <c r="DB79" s="8"/>
+      <c r="DB79" s="33"/>
       <c r="DC79" s="8"/>
       <c r="DD79" s="8"/>
       <c r="DE79" s="8"/>
@@ -18370,11 +18470,13 @@
       <c r="CW80" s="32">
         <v>9.7353051485010553</v>
       </c>
-      <c r="CX80" s="33"/>
+      <c r="CX80" s="32">
+        <v>8.8971241917830781</v>
+      </c>
       <c r="CY80" s="33"/>
       <c r="CZ80" s="33"/>
       <c r="DA80" s="33"/>
-      <c r="DB80" s="8"/>
+      <c r="DB80" s="33"/>
       <c r="DC80" s="8"/>
       <c r="DD80" s="8"/>
       <c r="DE80" s="8"/>
@@ -18749,11 +18851,13 @@
       <c r="CW81" s="32">
         <v>6.4151687512959938</v>
       </c>
-      <c r="CX81" s="33"/>
+      <c r="CX81" s="32">
+        <v>6.8926099203904272</v>
+      </c>
       <c r="CY81" s="33"/>
       <c r="CZ81" s="33"/>
       <c r="DA81" s="33"/>
-      <c r="DB81" s="8"/>
+      <c r="DB81" s="33"/>
       <c r="DC81" s="8"/>
       <c r="DD81" s="8"/>
       <c r="DE81" s="8"/>
@@ -18925,11 +19029,11 @@
       <c r="CU82" s="26"/>
       <c r="CV82" s="26"/>
       <c r="CW82" s="26"/>
-      <c r="CX82" s="34"/>
+      <c r="CX82" s="26"/>
       <c r="CY82" s="34"/>
       <c r="CZ82" s="34"/>
       <c r="DA82" s="34"/>
-      <c r="DB82" s="8"/>
+      <c r="DB82" s="34"/>
       <c r="DC82" s="8"/>
       <c r="DD82" s="8"/>
       <c r="DE82" s="8"/>
@@ -19304,11 +19408,13 @@
       <c r="CW83" s="32">
         <v>5.4505627561364491</v>
       </c>
-      <c r="CX83" s="33"/>
+      <c r="CX83" s="32">
+        <v>5.8501992776329246</v>
+      </c>
       <c r="CY83" s="33"/>
       <c r="CZ83" s="33"/>
       <c r="DA83" s="33"/>
-      <c r="DB83" s="8"/>
+      <c r="DB83" s="33"/>
       <c r="DC83" s="8"/>
       <c r="DD83" s="8"/>
       <c r="DE83" s="8"/>
@@ -19481,19 +19587,20 @@
       <c r="CU84" s="27"/>
       <c r="CV84" s="27"/>
       <c r="CW84" s="27"/>
-      <c r="CX84" s="31"/>
+      <c r="CX84" s="27"/>
       <c r="CY84" s="31"/>
       <c r="CZ84" s="31"/>
       <c r="DA84" s="31"/>
+      <c r="DB84" s="31"/>
     </row>
     <row r="85" spans="1:175" x14ac:dyDescent="0.2">
       <c r="A85" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="CX85" s="29"/>
       <c r="CY85" s="29"/>
       <c r="CZ85" s="29"/>
       <c r="DA85" s="29"/>
+      <c r="DB85" s="29"/>
     </row>
     <row r="86" spans="1:175" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B86" s="8"/>
@@ -19596,11 +19703,11 @@
       <c r="CU86" s="26"/>
       <c r="CV86" s="26"/>
       <c r="CW86" s="26"/>
-      <c r="CX86" s="34"/>
+      <c r="CX86" s="26"/>
       <c r="CY86" s="34"/>
       <c r="CZ86" s="34"/>
       <c r="DA86" s="34"/>
-      <c r="DB86" s="8"/>
+      <c r="DB86" s="34"/>
       <c r="DC86" s="8"/>
       <c r="DD86" s="8"/>
       <c r="DE86" s="8"/>
@@ -19772,11 +19879,11 @@
       <c r="CU87" s="26"/>
       <c r="CV87" s="26"/>
       <c r="CW87" s="26"/>
-      <c r="CX87" s="34"/>
+      <c r="CX87" s="26"/>
       <c r="CY87" s="34"/>
       <c r="CZ87" s="34"/>
       <c r="DA87" s="34"/>
-      <c r="DB87" s="8"/>
+      <c r="DB87" s="34"/>
       <c r="DC87" s="8"/>
       <c r="DD87" s="8"/>
       <c r="DE87" s="8"/>
@@ -19851,67 +19958,67 @@
       <c r="A88" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="CX88" s="29"/>
       <c r="CY88" s="29"/>
       <c r="CZ88" s="29"/>
       <c r="DA88" s="29"/>
+      <c r="DB88" s="29"/>
     </row>
     <row r="89" spans="1:175" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="CX89" s="29"/>
       <c r="CY89" s="29"/>
       <c r="CZ89" s="29"/>
       <c r="DA89" s="29"/>
+      <c r="DB89" s="29"/>
     </row>
     <row r="90" spans="1:175" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="CX90" s="29"/>
       <c r="CY90" s="29"/>
       <c r="CZ90" s="29"/>
       <c r="DA90" s="29"/>
+      <c r="DB90" s="29"/>
     </row>
     <row r="91" spans="1:175" x14ac:dyDescent="0.2">
-      <c r="CX91" s="29"/>
       <c r="CY91" s="29"/>
       <c r="CZ91" s="29"/>
       <c r="DA91" s="29"/>
+      <c r="DB91" s="29"/>
     </row>
     <row r="92" spans="1:175" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="CX92" s="29"/>
       <c r="CY92" s="29"/>
       <c r="CZ92" s="29"/>
       <c r="DA92" s="29"/>
+      <c r="DB92" s="29"/>
     </row>
     <row r="93" spans="1:175" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="CX93" s="29"/>
       <c r="CY93" s="29"/>
       <c r="CZ93" s="29"/>
       <c r="DA93" s="29"/>
+      <c r="DB93" s="29"/>
     </row>
     <row r="94" spans="1:175" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="CX94" s="29"/>
       <c r="CY94" s="29"/>
       <c r="CZ94" s="29"/>
       <c r="DA94" s="29"/>
+      <c r="DB94" s="29"/>
     </row>
     <row r="95" spans="1:175" x14ac:dyDescent="0.2">
-      <c r="CX95" s="29"/>
       <c r="CY95" s="29"/>
       <c r="CZ95" s="29"/>
       <c r="DA95" s="29"/>
+      <c r="DB95" s="29"/>
     </row>
     <row r="96" spans="1:175" x14ac:dyDescent="0.2">
       <c r="A96" s="3"/>
@@ -20065,10 +20172,13 @@
       <c r="CU96" s="23"/>
       <c r="CV96" s="23"/>
       <c r="CW96" s="23"/>
-      <c r="CX96" s="30"/>
+      <c r="CX96" s="23" t="s">
+        <v>63</v>
+      </c>
       <c r="CY96" s="30"/>
       <c r="CZ96" s="30"/>
       <c r="DA96" s="30"/>
+      <c r="DB96" s="30"/>
     </row>
     <row r="97" spans="1:175" x14ac:dyDescent="0.2">
       <c r="A97" s="4" t="s">
@@ -20374,17 +20484,20 @@
       <c r="CW97" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="CX97" s="31"/>
+      <c r="CX97" s="24" t="s">
+        <v>2</v>
+      </c>
       <c r="CY97" s="31"/>
       <c r="CZ97" s="31"/>
       <c r="DA97" s="31"/>
+      <c r="DB97" s="31"/>
     </row>
     <row r="98" spans="1:175" ht="10.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="6"/>
-      <c r="CX98" s="29"/>
       <c r="CY98" s="29"/>
       <c r="CZ98" s="29"/>
       <c r="DA98" s="29"/>
+      <c r="DB98" s="29"/>
     </row>
     <row r="99" spans="1:175" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
@@ -20690,11 +20803,13 @@
       <c r="CW99" s="32">
         <v>3.7927321752196548</v>
       </c>
-      <c r="CX99" s="33"/>
+      <c r="CX99" s="32">
+        <v>0.28772588745691507</v>
+      </c>
       <c r="CY99" s="33"/>
       <c r="CZ99" s="33"/>
       <c r="DA99" s="33"/>
-      <c r="DB99" s="8"/>
+      <c r="DB99" s="33"/>
       <c r="DC99" s="8"/>
       <c r="DD99" s="8"/>
       <c r="DE99" s="8"/>
@@ -21069,11 +21184,13 @@
       <c r="CW100" s="32">
         <v>-6.1365886567613046</v>
       </c>
-      <c r="CX100" s="33"/>
+      <c r="CX100" s="32">
+        <v>3.0541712181860277</v>
+      </c>
       <c r="CY100" s="33"/>
       <c r="CZ100" s="33"/>
       <c r="DA100" s="33"/>
-      <c r="DB100" s="8"/>
+      <c r="DB100" s="33"/>
       <c r="DC100" s="8"/>
       <c r="DD100" s="8"/>
       <c r="DE100" s="8"/>
@@ -21448,11 +21565,13 @@
       <c r="CW101" s="32">
         <v>-1.0533477687317543</v>
       </c>
-      <c r="CX101" s="33"/>
+      <c r="CX101" s="32">
+        <v>12.25860284969977</v>
+      </c>
       <c r="CY101" s="33"/>
       <c r="CZ101" s="33"/>
       <c r="DA101" s="33"/>
-      <c r="DB101" s="8"/>
+      <c r="DB101" s="33"/>
       <c r="DC101" s="8"/>
       <c r="DD101" s="8"/>
       <c r="DE101" s="8"/>
@@ -21827,11 +21946,13 @@
       <c r="CW102" s="32">
         <v>0.11345086296911688</v>
       </c>
-      <c r="CX102" s="33"/>
+      <c r="CX102" s="32">
+        <v>2.7208224282392734</v>
+      </c>
       <c r="CY102" s="33"/>
       <c r="CZ102" s="33"/>
       <c r="DA102" s="33"/>
-      <c r="DB102" s="8"/>
+      <c r="DB102" s="33"/>
       <c r="DC102" s="8"/>
       <c r="DD102" s="8"/>
       <c r="DE102" s="8"/>
@@ -22206,11 +22327,13 @@
       <c r="CW103" s="32">
         <v>-1.9626811850934303</v>
       </c>
-      <c r="CX103" s="33"/>
+      <c r="CX103" s="32">
+        <v>3.0911224344107495</v>
+      </c>
       <c r="CY103" s="33"/>
       <c r="CZ103" s="33"/>
       <c r="DA103" s="33"/>
-      <c r="DB103" s="8"/>
+      <c r="DB103" s="33"/>
       <c r="DC103" s="8"/>
       <c r="DD103" s="8"/>
       <c r="DE103" s="8"/>
@@ -22585,11 +22708,13 @@
       <c r="CW104" s="32">
         <v>5.6483077399349497</v>
       </c>
-      <c r="CX104" s="33"/>
+      <c r="CX104" s="32">
+        <v>5.6947308716537322</v>
+      </c>
       <c r="CY104" s="33"/>
       <c r="CZ104" s="33"/>
       <c r="DA104" s="33"/>
-      <c r="DB104" s="8"/>
+      <c r="DB104" s="33"/>
       <c r="DC104" s="8"/>
       <c r="DD104" s="8"/>
       <c r="DE104" s="8"/>
@@ -22964,11 +23089,13 @@
       <c r="CW105" s="32">
         <v>6.0058621655516049</v>
       </c>
-      <c r="CX105" s="33"/>
+      <c r="CX105" s="32">
+        <v>3.5374974360975955</v>
+      </c>
       <c r="CY105" s="33"/>
       <c r="CZ105" s="33"/>
       <c r="DA105" s="33"/>
-      <c r="DB105" s="8"/>
+      <c r="DB105" s="33"/>
       <c r="DC105" s="8"/>
       <c r="DD105" s="8"/>
       <c r="DE105" s="8"/>
@@ -23343,11 +23470,13 @@
       <c r="CW106" s="32">
         <v>3.5428482945700779</v>
       </c>
-      <c r="CX106" s="33"/>
+      <c r="CX106" s="32">
+        <v>5.6788768945325927</v>
+      </c>
       <c r="CY106" s="33"/>
       <c r="CZ106" s="33"/>
       <c r="DA106" s="33"/>
-      <c r="DB106" s="8"/>
+      <c r="DB106" s="33"/>
       <c r="DC106" s="8"/>
       <c r="DD106" s="8"/>
       <c r="DE106" s="8"/>
@@ -23722,11 +23851,13 @@
       <c r="CW107" s="32">
         <v>6.9813940197132212</v>
       </c>
-      <c r="CX107" s="33"/>
+      <c r="CX107" s="32">
+        <v>5.4334607994919395</v>
+      </c>
       <c r="CY107" s="33"/>
       <c r="CZ107" s="33"/>
       <c r="DA107" s="33"/>
-      <c r="DB107" s="8"/>
+      <c r="DB107" s="33"/>
       <c r="DC107" s="8"/>
       <c r="DD107" s="8"/>
       <c r="DE107" s="8"/>
@@ -24101,11 +24232,13 @@
       <c r="CW108" s="32">
         <v>6.6324016893898374</v>
       </c>
-      <c r="CX108" s="33"/>
+      <c r="CX108" s="32">
+        <v>6.7004239138229451</v>
+      </c>
       <c r="CY108" s="33"/>
       <c r="CZ108" s="33"/>
       <c r="DA108" s="33"/>
-      <c r="DB108" s="8"/>
+      <c r="DB108" s="33"/>
       <c r="DC108" s="8"/>
       <c r="DD108" s="8"/>
       <c r="DE108" s="8"/>
@@ -24480,11 +24613,13 @@
       <c r="CW109" s="32">
         <v>7.0804187336179751</v>
       </c>
-      <c r="CX109" s="33"/>
+      <c r="CX109" s="32">
+        <v>4.2472837968456076</v>
+      </c>
       <c r="CY109" s="33"/>
       <c r="CZ109" s="33"/>
       <c r="DA109" s="33"/>
-      <c r="DB109" s="8"/>
+      <c r="DB109" s="33"/>
       <c r="DC109" s="8"/>
       <c r="DD109" s="8"/>
       <c r="DE109" s="8"/>
@@ -24859,11 +24994,13 @@
       <c r="CW110" s="32">
         <v>3.9744610163546525</v>
       </c>
-      <c r="CX110" s="33"/>
+      <c r="CX110" s="32">
+        <v>4.0446280596069926</v>
+      </c>
       <c r="CY110" s="33"/>
       <c r="CZ110" s="33"/>
       <c r="DA110" s="33"/>
-      <c r="DB110" s="8"/>
+      <c r="DB110" s="33"/>
       <c r="DC110" s="8"/>
       <c r="DD110" s="8"/>
       <c r="DE110" s="8"/>
@@ -25035,11 +25172,11 @@
       <c r="CU111" s="26"/>
       <c r="CV111" s="26"/>
       <c r="CW111" s="26"/>
-      <c r="CX111" s="34"/>
+      <c r="CX111" s="26"/>
       <c r="CY111" s="34"/>
       <c r="CZ111" s="34"/>
       <c r="DA111" s="34"/>
-      <c r="DB111" s="8"/>
+      <c r="DB111" s="34"/>
       <c r="DC111" s="8"/>
       <c r="DD111" s="8"/>
       <c r="DE111" s="8"/>
@@ -25414,11 +25551,13 @@
       <c r="CW112" s="32">
         <v>3.7778645631406675</v>
       </c>
-      <c r="CX112" s="33"/>
+      <c r="CX112" s="32">
+        <v>3.0158187478206173</v>
+      </c>
       <c r="CY112" s="33"/>
       <c r="CZ112" s="33"/>
       <c r="DA112" s="33"/>
-      <c r="DB112" s="8"/>
+      <c r="DB112" s="33"/>
       <c r="DC112" s="8"/>
       <c r="DD112" s="8"/>
       <c r="DE112" s="8"/>
@@ -25591,19 +25730,20 @@
       <c r="CU113" s="27"/>
       <c r="CV113" s="27"/>
       <c r="CW113" s="27"/>
-      <c r="CX113" s="31"/>
+      <c r="CX113" s="27"/>
       <c r="CY113" s="31"/>
       <c r="CZ113" s="31"/>
       <c r="DA113" s="31"/>
+      <c r="DB113" s="31"/>
     </row>
     <row r="114" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A114" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="CX114" s="29"/>
       <c r="CY114" s="29"/>
       <c r="CZ114" s="29"/>
       <c r="DA114" s="29"/>
+      <c r="DB114" s="29"/>
     </row>
     <row r="115" spans="1:179" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B115" s="8"/>
@@ -25710,7 +25850,7 @@
       <c r="CY115" s="26"/>
       <c r="CZ115" s="35"/>
       <c r="DA115" s="35"/>
-      <c r="DB115" s="8"/>
+      <c r="DB115" s="26"/>
       <c r="DC115" s="8"/>
       <c r="DD115" s="8"/>
       <c r="DE115" s="8"/>
@@ -25886,7 +26026,7 @@
       <c r="CY116" s="26"/>
       <c r="CZ116" s="35"/>
       <c r="DA116" s="35"/>
-      <c r="DB116" s="8"/>
+      <c r="DB116" s="26"/>
       <c r="DC116" s="8"/>
       <c r="DD116" s="8"/>
       <c r="DE116" s="8"/>
@@ -26140,6 +26280,9 @@
       <c r="CY124" s="23"/>
       <c r="CZ124" s="23"/>
       <c r="DA124" s="23"/>
+      <c r="DB124" s="23">
+        <v>2026</v>
+      </c>
     </row>
     <row r="125" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A125" s="4" t="s">
@@ -26456,6 +26599,9 @@
       </c>
       <c r="DA125" s="24" t="s">
         <v>5</v>
+      </c>
+      <c r="DB125" s="24" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="126" spans="1:179" ht="10.9" customHeight="1" x14ac:dyDescent="0.2">
@@ -26777,7 +26923,9 @@
       <c r="DA127" s="32">
         <v>131.86778373265545</v>
       </c>
-      <c r="DB127" s="8"/>
+      <c r="DB127" s="32">
+        <v>133.11486788395311</v>
+      </c>
       <c r="DC127" s="8"/>
       <c r="DD127" s="8"/>
       <c r="DE127" s="8"/>
@@ -27168,7 +27316,9 @@
       <c r="DA128" s="32">
         <v>179.64199174509974</v>
       </c>
-      <c r="DB128" s="8"/>
+      <c r="DB128" s="32">
+        <v>179.82769105344306</v>
+      </c>
       <c r="DC128" s="8"/>
       <c r="DD128" s="8"/>
       <c r="DE128" s="8"/>
@@ -27559,7 +27709,9 @@
       <c r="DA129" s="32">
         <v>117.76800384210829</v>
       </c>
-      <c r="DB129" s="8"/>
+      <c r="DB129" s="32">
+        <v>120.13131886305874</v>
+      </c>
       <c r="DC129" s="8"/>
       <c r="DD129" s="8"/>
       <c r="DE129" s="8"/>
@@ -27950,7 +28102,9 @@
       <c r="DA130" s="32">
         <v>125.86725529260727</v>
       </c>
-      <c r="DB130" s="8"/>
+      <c r="DB130" s="32">
+        <v>120.18253008179754</v>
+      </c>
       <c r="DC130" s="8"/>
       <c r="DD130" s="8"/>
       <c r="DE130" s="8"/>
@@ -28341,7 +28495,9 @@
       <c r="DA131" s="32">
         <v>122.79243000357187</v>
       </c>
-      <c r="DB131" s="8"/>
+      <c r="DB131" s="32">
+        <v>128.86312316991368</v>
+      </c>
       <c r="DC131" s="8"/>
       <c r="DD131" s="8"/>
       <c r="DE131" s="8"/>
@@ -28732,7 +28888,9 @@
       <c r="DA132" s="32">
         <v>124.99785489223083</v>
       </c>
-      <c r="DB132" s="8"/>
+      <c r="DB132" s="32">
+        <v>122.77660735459482</v>
+      </c>
       <c r="DC132" s="8"/>
       <c r="DD132" s="8"/>
       <c r="DE132" s="8"/>
@@ -29123,7 +29281,9 @@
       <c r="DA133" s="32">
         <v>126.90688111505668</v>
       </c>
-      <c r="DB133" s="8"/>
+      <c r="DB133" s="32">
+        <v>137.80396639177681</v>
+      </c>
       <c r="DC133" s="8"/>
       <c r="DD133" s="8"/>
       <c r="DE133" s="8"/>
@@ -29514,7 +29674,9 @@
       <c r="DA134" s="32">
         <v>99.235385806528512</v>
       </c>
-      <c r="DB134" s="8"/>
+      <c r="DB134" s="32">
+        <v>107.18399324950228</v>
+      </c>
       <c r="DC134" s="8"/>
       <c r="DD134" s="8"/>
       <c r="DE134" s="8"/>
@@ -29905,7 +30067,9 @@
       <c r="DA135" s="32">
         <v>117.50299598526549</v>
       </c>
-      <c r="DB135" s="8"/>
+      <c r="DB135" s="32">
+        <v>120.35498636349908</v>
+      </c>
       <c r="DC135" s="8"/>
       <c r="DD135" s="8"/>
       <c r="DE135" s="8"/>
@@ -30296,7 +30460,9 @@
       <c r="DA136" s="32">
         <v>114.18732657888424</v>
       </c>
-      <c r="DB136" s="8"/>
+      <c r="DB136" s="32">
+        <v>120.37896764805924</v>
+      </c>
       <c r="DC136" s="8"/>
       <c r="DD136" s="8"/>
       <c r="DE136" s="8"/>
@@ -30687,7 +30853,9 @@
       <c r="DA137" s="32">
         <v>130.926626431069</v>
       </c>
-      <c r="DB137" s="8"/>
+      <c r="DB137" s="32">
+        <v>135.83333333333334</v>
+      </c>
       <c r="DC137" s="8"/>
       <c r="DD137" s="8"/>
       <c r="DE137" s="8"/>
@@ -31078,7 +31246,9 @@
       <c r="DA138" s="32">
         <v>115.80114901676801</v>
       </c>
-      <c r="DB138" s="8"/>
+      <c r="DB138" s="32">
+        <v>131.73625706296522</v>
+      </c>
       <c r="DC138" s="8"/>
       <c r="DD138" s="8"/>
       <c r="DE138" s="8"/>
@@ -31258,7 +31428,7 @@
       <c r="CY139" s="26"/>
       <c r="CZ139" s="26"/>
       <c r="DA139" s="26"/>
-      <c r="DB139" s="8"/>
+      <c r="DB139" s="26"/>
       <c r="DC139" s="8"/>
       <c r="DD139" s="8"/>
       <c r="DE139" s="8"/>
@@ -31649,7 +31819,9 @@
       <c r="DA140" s="32">
         <v>125.75245526872317</v>
       </c>
-      <c r="DB140" s="8"/>
+      <c r="DB140" s="32">
+        <v>130.06285010024203</v>
+      </c>
       <c r="DC140" s="8"/>
       <c r="DD140" s="8"/>
       <c r="DE140" s="8"/>
@@ -31830,6 +32002,7 @@
       <c r="CY141" s="27"/>
       <c r="CZ141" s="27"/>
       <c r="DA141" s="27"/>
+      <c r="DB141" s="27"/>
     </row>
     <row r="142" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A142" s="12" t="s">
@@ -32024,6 +32197,9 @@
       <c r="CY153" s="23"/>
       <c r="CZ153" s="23"/>
       <c r="DA153" s="23"/>
+      <c r="DB153" s="23">
+        <v>2026</v>
+      </c>
     </row>
     <row r="154" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A154" s="4" t="s">
@@ -32340,6 +32516,9 @@
       </c>
       <c r="DA154" s="24" t="s">
         <v>5</v>
+      </c>
+      <c r="DB154" s="24" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="155" spans="1:179" ht="10.9" customHeight="1" x14ac:dyDescent="0.2">
@@ -32661,7 +32840,9 @@
       <c r="DA156" s="32">
         <v>37.35495101165894</v>
       </c>
-      <c r="DB156" s="8"/>
+      <c r="DB156" s="32">
+        <v>32.617855510780672</v>
+      </c>
       <c r="DC156" s="8"/>
       <c r="DD156" s="8"/>
       <c r="DE156" s="8"/>
@@ -33052,7 +33233,9 @@
       <c r="DA157" s="32">
         <v>1.9897456335966761</v>
       </c>
-      <c r="DB157" s="8"/>
+      <c r="DB157" s="32">
+        <v>1.8035476286195591</v>
+      </c>
       <c r="DC157" s="8"/>
       <c r="DD157" s="8"/>
       <c r="DE157" s="8"/>
@@ -33443,7 +33626,9 @@
       <c r="DA158" s="32">
         <v>1.5676254952267776</v>
       </c>
-      <c r="DB158" s="8"/>
+      <c r="DB158" s="32">
+        <v>1.3754731629479835</v>
+      </c>
       <c r="DC158" s="8"/>
       <c r="DD158" s="8"/>
       <c r="DE158" s="8"/>
@@ -33834,7 +34019,9 @@
       <c r="DA159" s="32">
         <v>10.450112164051506</v>
       </c>
-      <c r="DB159" s="8"/>
+      <c r="DB159" s="32">
+        <v>10.959719702513523</v>
+      </c>
       <c r="DC159" s="8"/>
       <c r="DD159" s="8"/>
       <c r="DE159" s="8"/>
@@ -34225,7 +34412,9 @@
       <c r="DA160" s="32">
         <v>2.4403664072674704</v>
       </c>
-      <c r="DB160" s="8"/>
+      <c r="DB160" s="32">
+        <v>2.3748278876814086</v>
+      </c>
       <c r="DC160" s="8"/>
       <c r="DD160" s="8"/>
       <c r="DE160" s="8"/>
@@ -34616,7 +34805,9 @@
       <c r="DA161" s="32">
         <v>4.4588421426957927</v>
       </c>
-      <c r="DB161" s="8"/>
+      <c r="DB161" s="32">
+        <v>4.5933686278660755</v>
+      </c>
       <c r="DC161" s="8"/>
       <c r="DD161" s="8"/>
       <c r="DE161" s="8"/>
@@ -35007,7 +35198,9 @@
       <c r="DA162" s="32">
         <v>8.2180309363383532</v>
       </c>
-      <c r="DB162" s="8"/>
+      <c r="DB162" s="32">
+        <v>10.920402074268493</v>
+      </c>
       <c r="DC162" s="8"/>
       <c r="DD162" s="8"/>
       <c r="DE162" s="8"/>
@@ -35398,7 +35591,9 @@
       <c r="DA163" s="32">
         <v>2.4102637552467896</v>
       </c>
-      <c r="DB163" s="8"/>
+      <c r="DB163" s="32">
+        <v>2.7824009136202443</v>
+      </c>
       <c r="DC163" s="8"/>
       <c r="DD163" s="8"/>
       <c r="DE163" s="8"/>
@@ -35789,7 +35984,9 @@
       <c r="DA164" s="32">
         <v>1.9207835906935355</v>
       </c>
-      <c r="DB164" s="8"/>
+      <c r="DB164" s="32">
+        <v>1.917862352745934</v>
+      </c>
       <c r="DC164" s="8"/>
       <c r="DD164" s="8"/>
       <c r="DE164" s="8"/>
@@ -36180,7 +36377,9 @@
       <c r="DA165" s="32">
         <v>4.9640629602150677</v>
       </c>
-      <c r="DB165" s="8"/>
+      <c r="DB165" s="32">
+        <v>5.5261147905211487</v>
+      </c>
       <c r="DC165" s="8"/>
       <c r="DD165" s="8"/>
       <c r="DE165" s="8"/>
@@ -36571,7 +36770,9 @@
       <c r="DA166" s="32">
         <v>9.1027974592063732</v>
       </c>
-      <c r="DB166" s="8"/>
+      <c r="DB166" s="32">
+        <v>10.845627002812328</v>
+      </c>
       <c r="DC166" s="8"/>
       <c r="DD166" s="8"/>
       <c r="DE166" s="8"/>
@@ -36962,7 +37163,9 @@
       <c r="DA167" s="32">
         <v>15.122418443802719</v>
       </c>
-      <c r="DB167" s="8"/>
+      <c r="DB167" s="32">
+        <v>14.282800345622624</v>
+      </c>
       <c r="DC167" s="8"/>
       <c r="DD167" s="8"/>
       <c r="DE167" s="8"/>
@@ -37142,7 +37345,7 @@
       <c r="CY168" s="26"/>
       <c r="CZ168" s="26"/>
       <c r="DA168" s="26"/>
-      <c r="DB168" s="8"/>
+      <c r="DB168" s="26"/>
       <c r="DC168" s="8"/>
       <c r="DD168" s="8"/>
       <c r="DE168" s="8"/>
@@ -37533,7 +37736,9 @@
       <c r="DA169" s="32">
         <v>100</v>
       </c>
-      <c r="DB169" s="8"/>
+      <c r="DB169" s="32">
+        <v>100</v>
+      </c>
       <c r="DC169" s="8"/>
       <c r="DD169" s="8"/>
       <c r="DE169" s="8"/>
@@ -37714,6 +37919,7 @@
       <c r="CY170" s="27"/>
       <c r="CZ170" s="27"/>
       <c r="DA170" s="27"/>
+      <c r="DB170" s="27"/>
     </row>
     <row r="171" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A171" s="12" t="s">
@@ -37825,7 +38031,7 @@
       <c r="CY172" s="26"/>
       <c r="CZ172" s="26"/>
       <c r="DA172" s="26"/>
-      <c r="DB172" s="8"/>
+      <c r="DB172" s="26"/>
       <c r="DC172" s="8"/>
       <c r="DD172" s="8"/>
       <c r="DE172" s="8"/>
@@ -38005,7 +38211,7 @@
       <c r="CY173" s="26"/>
       <c r="CZ173" s="26"/>
       <c r="DA173" s="26"/>
-      <c r="DB173" s="8"/>
+      <c r="DB173" s="26"/>
       <c r="DC173" s="8"/>
       <c r="DD173" s="8"/>
       <c r="DE173" s="8"/>
@@ -38268,6 +38474,9 @@
       <c r="CY182" s="23"/>
       <c r="CZ182" s="23"/>
       <c r="DA182" s="23"/>
+      <c r="DB182" s="23">
+        <v>2026</v>
+      </c>
     </row>
     <row r="183" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A183" s="4" t="s">
@@ -38584,6 +38793,9 @@
       </c>
       <c r="DA183" s="24" t="s">
         <v>5</v>
+      </c>
+      <c r="DB183" s="24" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="184" spans="1:179" ht="10.9" customHeight="1" x14ac:dyDescent="0.2">
@@ -38905,7 +39117,9 @@
       <c r="DA185" s="32">
         <v>35.622626491414316</v>
       </c>
-      <c r="DB185" s="8"/>
+      <c r="DB185" s="32">
+        <v>31.870003098289786</v>
+      </c>
       <c r="DC185" s="8"/>
       <c r="DD185" s="8"/>
       <c r="DE185" s="8"/>
@@ -39296,7 +39510,9 @@
       <c r="DA186" s="32">
         <v>1.3928558482030335</v>
       </c>
-      <c r="DB186" s="8"/>
+      <c r="DB186" s="32">
+        <v>1.3044406203273744</v>
+      </c>
       <c r="DC186" s="8"/>
       <c r="DD186" s="8"/>
       <c r="DE186" s="8"/>
@@ -39687,7 +39903,9 @@
       <c r="DA187" s="32">
         <v>1.6739075855519421</v>
       </c>
-      <c r="DB187" s="8"/>
+      <c r="DB187" s="32">
+        <v>1.4891866792317539</v>
+      </c>
       <c r="DC187" s="8"/>
       <c r="DD187" s="8"/>
       <c r="DE187" s="8"/>
@@ -40078,7 +40296,9 @@
       <c r="DA188" s="32">
         <v>10.440580907306169</v>
       </c>
-      <c r="DB188" s="8"/>
+      <c r="DB188" s="32">
+        <v>11.860728675278406</v>
+      </c>
       <c r="DC188" s="8"/>
       <c r="DD188" s="8"/>
       <c r="DE188" s="8"/>
@@ -40469,7 +40689,9 @@
       <c r="DA189" s="32">
         <v>2.4991936999721429</v>
       </c>
-      <c r="DB189" s="8"/>
+      <c r="DB189" s="32">
+        <v>2.3969377427094405</v>
+      </c>
       <c r="DC189" s="8"/>
       <c r="DD189" s="8"/>
       <c r="DE189" s="8"/>
@@ -40860,7 +41082,9 @@
       <c r="DA190" s="32">
         <v>4.4857597563020342</v>
       </c>
-      <c r="DB190" s="8"/>
+      <c r="DB190" s="32">
+        <v>4.865964520227001</v>
+      </c>
       <c r="DC190" s="8"/>
       <c r="DD190" s="8"/>
       <c r="DE190" s="8"/>
@@ -41251,7 +41475,9 @@
       <c r="DA191" s="32">
         <v>8.1432744910178165</v>
       </c>
-      <c r="DB191" s="8"/>
+      <c r="DB191" s="32">
+        <v>10.306950193160123</v>
+      </c>
       <c r="DC191" s="8"/>
       <c r="DD191" s="8"/>
       <c r="DE191" s="8"/>
@@ -41642,7 +41868,9 @@
       <c r="DA192" s="32">
         <v>3.0543196119418572</v>
       </c>
-      <c r="DB192" s="8"/>
+      <c r="DB192" s="32">
+        <v>3.3763156416888469</v>
+      </c>
       <c r="DC192" s="8"/>
       <c r="DD192" s="8"/>
       <c r="DE192" s="8"/>
@@ -42033,7 +42261,9 @@
       <c r="DA193" s="32">
         <v>2.0556348418543737</v>
       </c>
-      <c r="DB193" s="8"/>
+      <c r="DB193" s="32">
+        <v>2.0725576167215798</v>
+      </c>
       <c r="DC193" s="8"/>
       <c r="DD193" s="8"/>
       <c r="DE193" s="8"/>
@@ -42424,7 +42654,9 @@
       <c r="DA194" s="32">
         <v>5.4668335274871662</v>
       </c>
-      <c r="DB194" s="8"/>
+      <c r="DB194" s="32">
+        <v>5.9706629295709055</v>
+      </c>
       <c r="DC194" s="8"/>
       <c r="DD194" s="8"/>
       <c r="DE194" s="8"/>
@@ -42815,7 +43047,9 @@
       <c r="DA195" s="32">
         <v>8.7430583183304122</v>
       </c>
-      <c r="DB195" s="8"/>
+      <c r="DB195" s="32">
+        <v>10.384882152956447</v>
+      </c>
       <c r="DC195" s="8"/>
       <c r="DD195" s="8"/>
       <c r="DE195" s="8"/>
@@ -43206,7 +43440,9 @@
       <c r="DA196" s="32">
         <v>16.421954920618724</v>
       </c>
-      <c r="DB196" s="8"/>
+      <c r="DB196" s="32">
+        <v>14.101370129838322</v>
+      </c>
       <c r="DC196" s="8"/>
       <c r="DD196" s="8"/>
       <c r="DE196" s="8"/>
@@ -43386,7 +43622,7 @@
       <c r="CY197" s="26"/>
       <c r="CZ197" s="26"/>
       <c r="DA197" s="26"/>
-      <c r="DB197" s="8"/>
+      <c r="DB197" s="26"/>
       <c r="DC197" s="8"/>
       <c r="DD197" s="8"/>
       <c r="DE197" s="8"/>
@@ -43777,7 +44013,9 @@
       <c r="DA198" s="32">
         <v>100</v>
       </c>
-      <c r="DB198" s="8"/>
+      <c r="DB198" s="32">
+        <v>100</v>
+      </c>
       <c r="DC198" s="8"/>
       <c r="DD198" s="8"/>
       <c r="DE198" s="8"/>
@@ -43958,6 +44196,7 @@
       <c r="CY199" s="27"/>
       <c r="CZ199" s="27"/>
       <c r="DA199" s="27"/>
+      <c r="DB199" s="27"/>
     </row>
     <row r="200" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A200" s="12" t="s">
@@ -44070,7 +44309,7 @@
       <c r="CY201" s="36"/>
       <c r="CZ201" s="36"/>
       <c r="DA201" s="36"/>
-      <c r="DB201" s="20"/>
+      <c r="DB201" s="36"/>
       <c r="DC201" s="20"/>
       <c r="DD201" s="20"/>
       <c r="DE201" s="20"/>
@@ -44150,6 +44389,7 @@
       <c r="CY202" s="29"/>
       <c r="CZ202" s="29"/>
       <c r="DA202" s="29"/>
+      <c r="DB202" s="28"/>
     </row>
     <row r="203" spans="1:179" x14ac:dyDescent="0.2">
       <c r="CT203" s="28"/>

</xml_diff>

<commit_message>
Q2 2026 SNA Update
</commit_message>
<xml_diff>
--- a/Data/National Accounts/PSA-02HFCE_2018PSNA_Qrt.xlsx
+++ b/Data/National Accounts/PSA-02HFCE_2018PSNA_Qrt.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Shared drives\QNAP\NAP Dissemination\As of May 2026\Tables\NAP Q1 2000 to Q1 2026\Qtr\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Shared drives\QNAP\NAP Dissemination\As of August 2026\Tables\NAP Q1 2000 to Q2 2026\Qtr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E40A17C-6613-41F7-A73A-5E7AE0B57C73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B520A11-6354-4D71-BABC-0AE46CD90C96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="794" xr2:uid="{736930C2-BFBB-46C3-AE9E-AECFC8C3145D}"/>
   </bookViews>
@@ -521,7 +521,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="932" uniqueCount="64">
   <si>
     <t>National Accounts of the Philippines</t>
   </si>
@@ -707,13 +707,13 @@
     <t>Percent Share, at Constant 2018 Prices</t>
   </si>
   <si>
-    <t>Q1 2000 to Q1 2026</t>
+    <t>2025 - 2026</t>
   </si>
   <si>
-    <t>As of May 2026</t>
+    <t>Q1 2000 to Q2 2026</t>
   </si>
   <si>
-    <t>2025 - 2026</t>
+    <t>As of August 2026</t>
   </si>
 </sst>
 </file>
@@ -1247,8 +1247,8 @@
     <col min="75" max="77" width="16.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="78" max="78" width="16.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="79" max="93" width="16.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="94" max="106" width="16.42578125" style="22" bestFit="1" customWidth="1"/>
-    <col min="107" max="16384" width="10" style="1"/>
+    <col min="94" max="107" width="16.42578125" style="22" bestFit="1" customWidth="1"/>
+    <col min="108" max="16384" width="10" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:179" x14ac:dyDescent="0.2">
@@ -1263,7 +1263,7 @@
     </row>
     <row r="3" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:179" x14ac:dyDescent="0.2">
@@ -1273,7 +1273,7 @@
     </row>
     <row r="6" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:179" x14ac:dyDescent="0.2">
@@ -1442,6 +1442,7 @@
       <c r="DB9" s="23">
         <v>2026</v>
       </c>
+      <c r="DC9" s="23"/>
     </row>
     <row r="10" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
@@ -1761,6 +1762,9 @@
       </c>
       <c r="DB10" s="24" t="s">
         <v>2</v>
+      </c>
+      <c r="DC10" s="24" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:179" ht="10.9" customHeight="1" x14ac:dyDescent="0.2">
@@ -2083,9 +2087,11 @@
         <v>2257594.2514206418</v>
       </c>
       <c r="DB12" s="25">
-        <v>1778620.7258560532</v>
-      </c>
-      <c r="DC12" s="8"/>
+        <v>1780849.5021926407</v>
+      </c>
+      <c r="DC12" s="25">
+        <v>2058217.46614084</v>
+      </c>
       <c r="DD12" s="8"/>
       <c r="DE12" s="8"/>
       <c r="DF12" s="8"/>
@@ -2476,9 +2482,11 @@
         <v>120252.82278633314</v>
       </c>
       <c r="DB13" s="25">
-        <v>98345.741683448505</v>
-      </c>
-      <c r="DC13" s="8"/>
+        <v>98404.506053292906</v>
+      </c>
+      <c r="DC13" s="25">
+        <v>88583.220711925562</v>
+      </c>
       <c r="DD13" s="8"/>
       <c r="DE13" s="8"/>
       <c r="DF13" s="8"/>
@@ -2869,9 +2877,11 @@
         <v>94741.452218738676</v>
       </c>
       <c r="DB14" s="25">
-        <v>75003.247061091388</v>
-      </c>
-      <c r="DC14" s="8"/>
+        <v>74660.902374091107</v>
+      </c>
+      <c r="DC14" s="25">
+        <v>57970.71664216894</v>
+      </c>
       <c r="DD14" s="8"/>
       <c r="DE14" s="8"/>
       <c r="DF14" s="8"/>
@@ -3262,9 +3272,11 @@
         <v>631565.8971390489</v>
       </c>
       <c r="DB15" s="25">
-        <v>597623.12105468463</v>
-      </c>
-      <c r="DC15" s="8"/>
+        <v>596954.41877003794</v>
+      </c>
+      <c r="DC15" s="25">
+        <v>796194.96285803744</v>
+      </c>
       <c r="DD15" s="8"/>
       <c r="DE15" s="8"/>
       <c r="DF15" s="8"/>
@@ -3655,9 +3667,11 @@
         <v>147486.66570831661</v>
       </c>
       <c r="DB16" s="25">
-        <v>129497.11240136674</v>
-      </c>
-      <c r="DC16" s="8"/>
+        <v>129990.33583773799</v>
+      </c>
+      <c r="DC16" s="25">
+        <v>129638.87097918091</v>
+      </c>
       <c r="DD16" s="8"/>
       <c r="DE16" s="8"/>
       <c r="DF16" s="8"/>
@@ -4048,9 +4062,11 @@
         <v>269475.82895237411</v>
       </c>
       <c r="DB17" s="25">
-        <v>250472.03487425239</v>
-      </c>
-      <c r="DC17" s="8"/>
+        <v>251185.654706598</v>
+      </c>
+      <c r="DC17" s="25">
+        <v>226844.92785009029</v>
+      </c>
       <c r="DD17" s="8"/>
       <c r="DE17" s="8"/>
       <c r="DF17" s="8"/>
@@ -4441,9 +4457,11 @@
         <v>496667.21270987199</v>
       </c>
       <c r="DB18" s="25">
-        <v>595479.16807577095</v>
-      </c>
-      <c r="DC18" s="8"/>
+        <v>593895.94045136345</v>
+      </c>
+      <c r="DC18" s="25">
+        <v>522412.1896321784</v>
+      </c>
       <c r="DD18" s="8"/>
       <c r="DE18" s="8"/>
       <c r="DF18" s="8"/>
@@ -4834,9 +4852,11 @@
         <v>145667.37342405706</v>
       </c>
       <c r="DB19" s="25">
-        <v>151721.68295889723</v>
-      </c>
-      <c r="DC19" s="8"/>
+        <v>151503.80112033547</v>
+      </c>
+      <c r="DC19" s="25">
+        <v>160555.98892234967</v>
+      </c>
       <c r="DD19" s="8"/>
       <c r="DE19" s="8"/>
       <c r="DF19" s="8"/>
@@ -5227,9 +5247,11 @@
         <v>116085.0135024778</v>
       </c>
       <c r="DB20" s="25">
-        <v>104579.21517266936</v>
-      </c>
-      <c r="DC20" s="8"/>
+        <v>104659.88991530363</v>
+      </c>
+      <c r="DC20" s="25">
+        <v>71377.365557757425</v>
+      </c>
       <c r="DD20" s="8"/>
       <c r="DE20" s="8"/>
       <c r="DF20" s="8"/>
@@ -5620,9 +5642,11 @@
         <v>300009.49537248426</v>
       </c>
       <c r="DB21" s="25">
-        <v>301333.79849671648</v>
-      </c>
-      <c r="DC21" s="8"/>
+        <v>300578.64207675576</v>
+      </c>
+      <c r="DC21" s="25">
+        <v>289228.62662580737</v>
+      </c>
       <c r="DD21" s="8"/>
       <c r="DE21" s="8"/>
       <c r="DF21" s="8"/>
@@ -6013,9 +6037,11 @@
         <v>550139.20937379065</v>
       </c>
       <c r="DB22" s="25">
-        <v>591401.75434679841</v>
-      </c>
-      <c r="DC22" s="8"/>
+        <v>592865.6798324649</v>
+      </c>
+      <c r="DC22" s="25">
+        <v>331836.13911109738</v>
+      </c>
       <c r="DD22" s="8"/>
       <c r="DE22" s="8"/>
       <c r="DF22" s="8"/>
@@ -6406,9 +6432,11 @@
         <v>913942.70429242158</v>
       </c>
       <c r="DB23" s="25">
-        <v>778827.55687577662</v>
-      </c>
-      <c r="DC23" s="8"/>
+        <v>778171.00851412956</v>
+      </c>
+      <c r="DC23" s="25">
+        <v>754238.1811308359</v>
+      </c>
       <c r="DD23" s="8"/>
       <c r="DE23" s="8"/>
       <c r="DF23" s="8"/>
@@ -6588,7 +6616,7 @@
       <c r="CZ24" s="26"/>
       <c r="DA24" s="26"/>
       <c r="DB24" s="26"/>
-      <c r="DC24" s="8"/>
+      <c r="DC24" s="26"/>
       <c r="DD24" s="8"/>
       <c r="DE24" s="8"/>
       <c r="DF24" s="8"/>
@@ -6979,9 +7007,11 @@
         <v>6043627.9269005563</v>
       </c>
       <c r="DB25" s="10">
-        <v>5452905.1588575263</v>
-      </c>
-      <c r="DC25" s="8"/>
+        <v>5453720.281844751</v>
+      </c>
+      <c r="DC25" s="10">
+        <v>5487098.6561622685</v>
+      </c>
       <c r="DD25" s="8"/>
       <c r="DE25" s="8"/>
       <c r="DF25" s="8"/>
@@ -7162,6 +7192,7 @@
       <c r="CZ26" s="27"/>
       <c r="DA26" s="27"/>
       <c r="DB26" s="27"/>
+      <c r="DC26" s="27"/>
     </row>
     <row r="27" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A27" s="12" t="s">
@@ -7274,7 +7305,7 @@
       <c r="CZ28" s="15"/>
       <c r="DA28" s="15"/>
       <c r="DB28" s="15"/>
-      <c r="DC28" s="8"/>
+      <c r="DC28" s="15"/>
       <c r="DD28" s="8"/>
       <c r="DE28" s="8"/>
       <c r="DF28" s="8"/>
@@ -7454,7 +7485,7 @@
       <c r="CZ29" s="17"/>
       <c r="DA29" s="17"/>
       <c r="DB29" s="17"/>
-      <c r="DC29" s="8"/>
+      <c r="DC29" s="17"/>
       <c r="DD29" s="8"/>
       <c r="DE29" s="8"/>
       <c r="DF29" s="8"/>
@@ -7540,7 +7571,7 @@
     </row>
     <row r="32" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="34" spans="1:179" x14ac:dyDescent="0.2">
@@ -7550,7 +7581,7 @@
     </row>
     <row r="35" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="36" spans="1:179" x14ac:dyDescent="0.2">
@@ -7719,6 +7750,7 @@
       <c r="DB38" s="23">
         <v>2026</v>
       </c>
+      <c r="DC38" s="23"/>
     </row>
     <row r="39" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
@@ -8038,6 +8070,9 @@
       </c>
       <c r="DB39" s="24" t="s">
         <v>2</v>
+      </c>
+      <c r="DC39" s="24" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="40" spans="1:179" ht="10.9" customHeight="1" x14ac:dyDescent="0.2">
@@ -8360,9 +8395,11 @@
         <v>1712013.4937564556</v>
       </c>
       <c r="DB41" s="25">
-        <v>1336154.8218690488</v>
-      </c>
-      <c r="DC41" s="18"/>
+        <v>1337829.1474887312</v>
+      </c>
+      <c r="DC41" s="25">
+        <v>1474396.4868965195</v>
+      </c>
       <c r="DD41" s="18"/>
       <c r="DE41" s="8"/>
       <c r="DF41" s="8"/>
@@ -8753,9 +8790,11 @@
         <v>66940.263586569476</v>
       </c>
       <c r="DB42" s="25">
-        <v>54688.87528240637</v>
-      </c>
-      <c r="DC42" s="18"/>
+        <v>54721.553436421556</v>
+      </c>
+      <c r="DC42" s="25">
+        <v>44521.969899765572</v>
+      </c>
       <c r="DD42" s="18"/>
       <c r="DE42" s="8"/>
       <c r="DF42" s="8"/>
@@ -9146,9 +9185,11 @@
         <v>80447.531696095204</v>
       </c>
       <c r="DB43" s="25">
-        <v>62434.382449917008</v>
-      </c>
-      <c r="DC43" s="18"/>
+        <v>62149.40706611178</v>
+      </c>
+      <c r="DC43" s="25">
+        <v>43943.727905410917</v>
+      </c>
       <c r="DD43" s="18"/>
       <c r="DE43" s="8"/>
       <c r="DF43" s="8"/>
@@ -9539,9 +9580,11 @@
         <v>501771.40644787182</v>
       </c>
       <c r="DB44" s="25">
-        <v>497262.88891400094</v>
-      </c>
-      <c r="DC44" s="18"/>
+        <v>496706.48334973835</v>
+      </c>
+      <c r="DC44" s="25">
+        <v>609382.27496379381</v>
+      </c>
       <c r="DD44" s="18"/>
       <c r="DE44" s="8"/>
       <c r="DF44" s="8"/>
@@ -9932,9 +9975,11 @@
         <v>120110.55217656854</v>
       </c>
       <c r="DB45" s="25">
-        <v>100491.98654809655</v>
-      </c>
-      <c r="DC45" s="18"/>
+        <v>100874.73641806586</v>
+      </c>
+      <c r="DC45" s="25">
+        <v>100045.44612950395</v>
+      </c>
       <c r="DD45" s="18"/>
       <c r="DE45" s="8"/>
       <c r="DF45" s="8"/>
@@ -10325,9 +10370,11 @@
         <v>215584.36277543131</v>
       </c>
       <c r="DB46" s="25">
-        <v>204006.31705912558</v>
-      </c>
-      <c r="DC46" s="18"/>
+        <v>204587.55142267546</v>
+      </c>
+      <c r="DC46" s="25">
+        <v>181823.8324297306</v>
+      </c>
       <c r="DD46" s="18"/>
       <c r="DE46" s="8"/>
       <c r="DF46" s="8"/>
@@ -10718,9 +10765,11 @@
         <v>391363.50081725052</v>
       </c>
       <c r="DB47" s="25">
-        <v>432120.48511203448</v>
-      </c>
-      <c r="DC47" s="18"/>
+        <v>430971.58666893281</v>
+      </c>
+      <c r="DC47" s="25">
+        <v>356283.62200209987</v>
+      </c>
       <c r="DD47" s="18"/>
       <c r="DE47" s="8"/>
       <c r="DF47" s="8"/>
@@ -11111,9 +11160,11 @@
         <v>146789.74867700256</v>
       </c>
       <c r="DB48" s="25">
-        <v>141552.55683161606</v>
-      </c>
-      <c r="DC48" s="18"/>
+        <v>141349.27849503219</v>
+      </c>
+      <c r="DC48" s="25">
+        <v>153529.31980295136</v>
+      </c>
       <c r="DD48" s="18"/>
       <c r="DE48" s="8"/>
       <c r="DF48" s="8"/>
@@ -11504,9 +11555,11 @@
         <v>98793.237167360829</v>
       </c>
       <c r="DB49" s="25">
-        <v>86892.299465529941</v>
-      </c>
-      <c r="DC49" s="18"/>
+        <v>86959.330126304252</v>
+      </c>
+      <c r="DC49" s="25">
+        <v>59323.875462414973</v>
+      </c>
       <c r="DD49" s="18"/>
       <c r="DE49" s="8"/>
       <c r="DF49" s="8"/>
@@ -11897,9 +11950,11 @@
         <v>262734.49458966724</v>
       </c>
       <c r="DB50" s="25">
-        <v>250320.96917270299</v>
-      </c>
-      <c r="DC50" s="18"/>
+        <v>249693.65325970354</v>
+      </c>
+      <c r="DC50" s="25">
+        <v>233600.03422705273</v>
+      </c>
       <c r="DD50" s="18"/>
       <c r="DE50" s="8"/>
       <c r="DF50" s="8"/>
@@ -12290,9 +12345,11 @@
         <v>420188.94427363185</v>
       </c>
       <c r="DB51" s="25">
-        <v>435387.79461113992</v>
-      </c>
-      <c r="DC51" s="18"/>
+        <v>436465.53116500482</v>
+      </c>
+      <c r="DC51" s="25">
+        <v>246355.58688284273</v>
+      </c>
       <c r="DD51" s="18"/>
       <c r="DE51" s="8"/>
       <c r="DF51" s="8"/>
@@ -12683,9 +12740,11 @@
         <v>789234.57327706018</v>
       </c>
       <c r="DB52" s="25">
-        <v>591202.12934509362</v>
-      </c>
-      <c r="DC52" s="18"/>
+        <v>590703.74843137653</v>
+      </c>
+      <c r="DC52" s="25">
+        <v>558989.98855918273</v>
+      </c>
       <c r="DD52" s="18"/>
       <c r="DE52" s="8"/>
       <c r="DF52" s="8"/>
@@ -12865,7 +12924,7 @@
       <c r="CZ53" s="26"/>
       <c r="DA53" s="26"/>
       <c r="DB53" s="26"/>
-      <c r="DC53" s="8"/>
+      <c r="DC53" s="26"/>
       <c r="DD53" s="8"/>
       <c r="DE53" s="8"/>
       <c r="DF53" s="8"/>
@@ -13256,9 +13315,11 @@
         <v>4805972.1092409659</v>
       </c>
       <c r="DB54" s="10">
-        <v>4192515.5066607129</v>
-      </c>
-      <c r="DC54" s="8"/>
+        <v>4193012.0073280982</v>
+      </c>
+      <c r="DC54" s="10">
+        <v>4062196.1651612697</v>
+      </c>
       <c r="DD54" s="8"/>
       <c r="DE54" s="8"/>
       <c r="DF54" s="8"/>
@@ -13439,6 +13500,7 @@
       <c r="CZ55" s="27"/>
       <c r="DA55" s="27"/>
       <c r="DB55" s="27"/>
+      <c r="DC55" s="27"/>
     </row>
     <row r="56" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A56" s="12" t="s">
@@ -13551,7 +13613,7 @@
       <c r="CZ57" s="26"/>
       <c r="DA57" s="26"/>
       <c r="DB57" s="26"/>
-      <c r="DC57" s="8"/>
+      <c r="DC57" s="26"/>
       <c r="DD57" s="8"/>
       <c r="DE57" s="8"/>
       <c r="DF57" s="8"/>
@@ -13731,7 +13793,7 @@
       <c r="CZ58" s="17"/>
       <c r="DA58" s="17"/>
       <c r="DB58" s="17"/>
-      <c r="DC58" s="8"/>
+      <c r="DC58" s="17"/>
       <c r="DD58" s="8"/>
       <c r="DE58" s="8"/>
       <c r="DF58" s="8"/>
@@ -13817,7 +13879,7 @@
     </row>
     <row r="61" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="CT61" s="28"/>
       <c r="CU61" s="28"/>
@@ -13827,6 +13889,7 @@
       <c r="CZ61" s="28"/>
       <c r="DA61" s="28"/>
       <c r="DB61" s="28"/>
+      <c r="DC61" s="28"/>
     </row>
     <row r="62" spans="1:179" x14ac:dyDescent="0.2">
       <c r="CT62" s="28"/>
@@ -13837,6 +13900,7 @@
       <c r="CZ62" s="28"/>
       <c r="DA62" s="28"/>
       <c r="DB62" s="28"/>
+      <c r="DC62" s="28"/>
     </row>
     <row r="63" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
@@ -13850,16 +13914,18 @@
       <c r="CZ63" s="28"/>
       <c r="DA63" s="28"/>
       <c r="DB63" s="28"/>
+      <c r="DC63" s="28"/>
     </row>
     <row r="64" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="CX64" s="28"/>
       <c r="CY64" s="28"/>
       <c r="CZ64" s="28"/>
       <c r="DA64" s="28"/>
       <c r="DB64" s="28"/>
+      <c r="DC64" s="28"/>
     </row>
     <row r="65" spans="1:175" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
@@ -13870,12 +13936,13 @@
       <c r="CZ65" s="29"/>
       <c r="DA65" s="29"/>
       <c r="DB65" s="29"/>
+      <c r="DC65" s="29"/>
     </row>
     <row r="66" spans="1:175" x14ac:dyDescent="0.2">
-      <c r="CY66" s="29"/>
       <c r="CZ66" s="29"/>
       <c r="DA66" s="29"/>
       <c r="DB66" s="29"/>
+      <c r="DC66" s="29"/>
     </row>
     <row r="67" spans="1:175" x14ac:dyDescent="0.2">
       <c r="A67" s="3"/>
@@ -14030,12 +14097,13 @@
       <c r="CV67" s="23"/>
       <c r="CW67" s="23"/>
       <c r="CX67" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="CY67" s="30"/>
+        <v>61</v>
+      </c>
+      <c r="CY67" s="23"/>
       <c r="CZ67" s="30"/>
       <c r="DA67" s="30"/>
       <c r="DB67" s="30"/>
+      <c r="DC67" s="30"/>
     </row>
     <row r="68" spans="1:175" x14ac:dyDescent="0.2">
       <c r="A68" s="4" t="s">
@@ -14344,17 +14412,20 @@
       <c r="CX68" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="CY68" s="31"/>
+      <c r="CY68" s="24" t="s">
+        <v>3</v>
+      </c>
       <c r="CZ68" s="31"/>
       <c r="DA68" s="31"/>
       <c r="DB68" s="31"/>
+      <c r="DC68" s="31"/>
     </row>
     <row r="69" spans="1:175" ht="10.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="6"/>
-      <c r="CY69" s="29"/>
       <c r="CZ69" s="29"/>
       <c r="DA69" s="29"/>
       <c r="DB69" s="29"/>
+      <c r="DC69" s="29"/>
     </row>
     <row r="70" spans="1:175" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
@@ -14661,13 +14732,15 @@
         <v>4.5040021672833319</v>
       </c>
       <c r="CX70" s="32">
-        <v>2.2521765703352798</v>
-      </c>
-      <c r="CY70" s="33"/>
+        <v>2.3803080084724684</v>
+      </c>
+      <c r="CY70" s="32">
+        <v>8.2679705361318412</v>
+      </c>
       <c r="CZ70" s="33"/>
       <c r="DA70" s="33"/>
       <c r="DB70" s="33"/>
-      <c r="DC70" s="8"/>
+      <c r="DC70" s="33"/>
       <c r="DD70" s="8"/>
       <c r="DE70" s="8"/>
       <c r="DF70" s="8"/>
@@ -15042,13 +15115,15 @@
         <v>-2.6867580532877611</v>
       </c>
       <c r="CX71" s="32">
-        <v>6.4741941354012198</v>
-      </c>
-      <c r="CY71" s="33"/>
+        <v>6.5378154861171112</v>
+      </c>
+      <c r="CY71" s="32">
+        <v>3.4416488326083083</v>
+      </c>
       <c r="CZ71" s="33"/>
       <c r="DA71" s="33"/>
       <c r="DB71" s="33"/>
-      <c r="DC71" s="8"/>
+      <c r="DC71" s="33"/>
       <c r="DD71" s="8"/>
       <c r="DE71" s="8"/>
       <c r="DF71" s="8"/>
@@ -15423,13 +15498,15 @@
         <v>0.85425742935640869</v>
       </c>
       <c r="CX72" s="32">
-        <v>15.005754421105095</v>
-      </c>
-      <c r="CY72" s="33"/>
+        <v>14.480822360917671</v>
+      </c>
+      <c r="CY72" s="32">
+        <v>11.067389945595821</v>
+      </c>
       <c r="CZ72" s="33"/>
       <c r="DA72" s="33"/>
       <c r="DB72" s="33"/>
-      <c r="DC72" s="8"/>
+      <c r="DC72" s="33"/>
       <c r="DD72" s="8"/>
       <c r="DE72" s="8"/>
       <c r="DF72" s="8"/>
@@ -15804,13 +15881,15 @@
         <v>2.8177282016049929</v>
       </c>
       <c r="CX73" s="32">
-        <v>6.6055781133850644</v>
-      </c>
-      <c r="CY73" s="33"/>
+        <v>6.4862932478418855</v>
+      </c>
+      <c r="CY73" s="32">
+        <v>11.484260027768144</v>
+      </c>
       <c r="CZ73" s="33"/>
       <c r="DA73" s="33"/>
       <c r="DB73" s="33"/>
-      <c r="DC73" s="8"/>
+      <c r="DC73" s="33"/>
       <c r="DD73" s="8"/>
       <c r="DE73" s="8"/>
       <c r="DF73" s="8"/>
@@ -16185,13 +16264,15 @@
         <v>6.2002573040501829E-2</v>
       </c>
       <c r="CX74" s="32">
-        <v>5.9292585985969453</v>
-      </c>
-      <c r="CY74" s="33"/>
+        <v>6.3327177334718812</v>
+      </c>
+      <c r="CY74" s="32">
+        <v>7.7735951606349403</v>
+      </c>
       <c r="CZ74" s="33"/>
       <c r="DA74" s="33"/>
       <c r="DB74" s="33"/>
-      <c r="DC74" s="8"/>
+      <c r="DC74" s="33"/>
       <c r="DD74" s="8"/>
       <c r="DE74" s="8"/>
       <c r="DF74" s="8"/>
@@ -16566,13 +16647,15 @@
         <v>8.517487380089122</v>
       </c>
       <c r="CX75" s="32">
-        <v>9.0823825021554256</v>
-      </c>
-      <c r="CY75" s="33"/>
+        <v>9.393169099757543</v>
+      </c>
+      <c r="CY75" s="32">
+        <v>14.327210698218011</v>
+      </c>
       <c r="CZ75" s="33"/>
       <c r="DA75" s="33"/>
       <c r="DB75" s="33"/>
-      <c r="DC75" s="8"/>
+      <c r="DC75" s="33"/>
       <c r="DD75" s="8"/>
       <c r="DE75" s="8"/>
       <c r="DF75" s="8"/>
@@ -16947,13 +17030,15 @@
         <v>7.0480931519140881</v>
       </c>
       <c r="CX76" s="32">
-        <v>6.748168166432734</v>
-      </c>
-      <c r="CY76" s="33"/>
+        <v>6.4643519428659033</v>
+      </c>
+      <c r="CY76" s="32">
+        <v>8.0402382831615569</v>
+      </c>
       <c r="CZ76" s="33"/>
       <c r="DA76" s="33"/>
       <c r="DB76" s="33"/>
-      <c r="DC76" s="8"/>
+      <c r="DC76" s="33"/>
       <c r="DD76" s="8"/>
       <c r="DE76" s="8"/>
       <c r="DF76" s="8"/>
@@ -17328,13 +17413,15 @@
         <v>4.245173815947993</v>
       </c>
       <c r="CX77" s="32">
-        <v>6.4283724753448723</v>
-      </c>
-      <c r="CY77" s="33"/>
+        <v>6.275534667209385</v>
+      </c>
+      <c r="CY77" s="32">
+        <v>6.4784458530672282</v>
+      </c>
       <c r="CZ77" s="33"/>
       <c r="DA77" s="33"/>
       <c r="DB77" s="33"/>
-      <c r="DC77" s="8"/>
+      <c r="DC77" s="33"/>
       <c r="DD77" s="8"/>
       <c r="DE77" s="8"/>
       <c r="DF77" s="8"/>
@@ -17709,13 +17796,15 @@
         <v>9.0856460685615872</v>
       </c>
       <c r="CX78" s="32">
-        <v>9.4690483265493128</v>
-      </c>
-      <c r="CY78" s="33"/>
+        <v>9.5534951957056933</v>
+      </c>
+      <c r="CY78" s="32">
+        <v>4.2612368733145161</v>
+      </c>
       <c r="CZ78" s="33"/>
       <c r="DA78" s="33"/>
       <c r="DB78" s="33"/>
-      <c r="DC78" s="8"/>
+      <c r="DC78" s="33"/>
       <c r="DD78" s="8"/>
       <c r="DE78" s="8"/>
       <c r="DF78" s="8"/>
@@ -18090,13 +18179,15 @@
         <v>9.8287101496879643</v>
       </c>
       <c r="CX79" s="32">
-        <v>9.8047587741586</v>
-      </c>
-      <c r="CY79" s="33"/>
+        <v>9.5295829759434412</v>
+      </c>
+      <c r="CY79" s="32">
+        <v>16.606873139897289</v>
+      </c>
       <c r="CZ79" s="33"/>
       <c r="DA79" s="33"/>
       <c r="DB79" s="33"/>
-      <c r="DC79" s="8"/>
+      <c r="DC79" s="33"/>
       <c r="DD79" s="8"/>
       <c r="DE79" s="8"/>
       <c r="DF79" s="8"/>
@@ -18471,13 +18562,15 @@
         <v>9.7353051485010553</v>
       </c>
       <c r="CX80" s="32">
-        <v>8.8971241917830781</v>
-      </c>
-      <c r="CY80" s="33"/>
+        <v>9.1666825321979246</v>
+      </c>
+      <c r="CY80" s="32">
+        <v>6.3842744872892467</v>
+      </c>
       <c r="CZ80" s="33"/>
       <c r="DA80" s="33"/>
       <c r="DB80" s="33"/>
-      <c r="DC80" s="8"/>
+      <c r="DC80" s="33"/>
       <c r="DD80" s="8"/>
       <c r="DE80" s="8"/>
       <c r="DF80" s="8"/>
@@ -18852,13 +18945,15 @@
         <v>6.4151687512959938</v>
       </c>
       <c r="CX81" s="32">
-        <v>6.8926099203904272</v>
-      </c>
-      <c r="CY81" s="33"/>
+        <v>6.8024998988640277</v>
+      </c>
+      <c r="CY81" s="32">
+        <v>9.6601117698580339</v>
+      </c>
       <c r="CZ81" s="33"/>
       <c r="DA81" s="33"/>
       <c r="DB81" s="33"/>
-      <c r="DC81" s="8"/>
+      <c r="DC81" s="33"/>
       <c r="DD81" s="8"/>
       <c r="DE81" s="8"/>
       <c r="DF81" s="8"/>
@@ -19030,11 +19125,11 @@
       <c r="CV82" s="26"/>
       <c r="CW82" s="26"/>
       <c r="CX82" s="26"/>
-      <c r="CY82" s="34"/>
+      <c r="CY82" s="26"/>
       <c r="CZ82" s="34"/>
       <c r="DA82" s="34"/>
       <c r="DB82" s="34"/>
-      <c r="DC82" s="8"/>
+      <c r="DC82" s="34"/>
       <c r="DD82" s="8"/>
       <c r="DE82" s="8"/>
       <c r="DF82" s="8"/>
@@ -19409,13 +19504,15 @@
         <v>5.4505627561364491</v>
       </c>
       <c r="CX83" s="32">
-        <v>5.8501992776329246</v>
-      </c>
-      <c r="CY83" s="33"/>
+        <v>5.8660222065340974</v>
+      </c>
+      <c r="CY83" s="32">
+        <v>9.2548995137978096</v>
+      </c>
       <c r="CZ83" s="33"/>
       <c r="DA83" s="33"/>
       <c r="DB83" s="33"/>
-      <c r="DC83" s="8"/>
+      <c r="DC83" s="33"/>
       <c r="DD83" s="8"/>
       <c r="DE83" s="8"/>
       <c r="DF83" s="8"/>
@@ -19588,19 +19685,20 @@
       <c r="CV84" s="27"/>
       <c r="CW84" s="27"/>
       <c r="CX84" s="27"/>
-      <c r="CY84" s="31"/>
+      <c r="CY84" s="27"/>
       <c r="CZ84" s="31"/>
       <c r="DA84" s="31"/>
       <c r="DB84" s="31"/>
+      <c r="DC84" s="31"/>
     </row>
     <row r="85" spans="1:175" x14ac:dyDescent="0.2">
       <c r="A85" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="CY85" s="29"/>
       <c r="CZ85" s="29"/>
       <c r="DA85" s="29"/>
       <c r="DB85" s="29"/>
+      <c r="DC85" s="29"/>
     </row>
     <row r="86" spans="1:175" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B86" s="8"/>
@@ -19704,11 +19802,11 @@
       <c r="CV86" s="26"/>
       <c r="CW86" s="26"/>
       <c r="CX86" s="26"/>
-      <c r="CY86" s="34"/>
+      <c r="CY86" s="26"/>
       <c r="CZ86" s="34"/>
       <c r="DA86" s="34"/>
       <c r="DB86" s="34"/>
-      <c r="DC86" s="8"/>
+      <c r="DC86" s="34"/>
       <c r="DD86" s="8"/>
       <c r="DE86" s="8"/>
       <c r="DF86" s="8"/>
@@ -19880,11 +19978,11 @@
       <c r="CV87" s="26"/>
       <c r="CW87" s="26"/>
       <c r="CX87" s="26"/>
-      <c r="CY87" s="34"/>
+      <c r="CY87" s="26"/>
       <c r="CZ87" s="34"/>
       <c r="DA87" s="34"/>
       <c r="DB87" s="34"/>
-      <c r="DC87" s="8"/>
+      <c r="DC87" s="34"/>
       <c r="DD87" s="8"/>
       <c r="DE87" s="8"/>
       <c r="DF87" s="8"/>
@@ -19958,67 +20056,67 @@
       <c r="A88" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="CY88" s="29"/>
       <c r="CZ88" s="29"/>
       <c r="DA88" s="29"/>
       <c r="DB88" s="29"/>
+      <c r="DC88" s="29"/>
     </row>
     <row r="89" spans="1:175" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="CY89" s="29"/>
       <c r="CZ89" s="29"/>
       <c r="DA89" s="29"/>
       <c r="DB89" s="29"/>
+      <c r="DC89" s="29"/>
     </row>
     <row r="90" spans="1:175" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="CY90" s="29"/>
+        <v>63</v>
+      </c>
       <c r="CZ90" s="29"/>
       <c r="DA90" s="29"/>
       <c r="DB90" s="29"/>
+      <c r="DC90" s="29"/>
     </row>
     <row r="91" spans="1:175" x14ac:dyDescent="0.2">
-      <c r="CY91" s="29"/>
       <c r="CZ91" s="29"/>
       <c r="DA91" s="29"/>
       <c r="DB91" s="29"/>
+      <c r="DC91" s="29"/>
     </row>
     <row r="92" spans="1:175" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="CY92" s="29"/>
       <c r="CZ92" s="29"/>
       <c r="DA92" s="29"/>
       <c r="DB92" s="29"/>
+      <c r="DC92" s="29"/>
     </row>
     <row r="93" spans="1:175" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="CY93" s="29"/>
+        <v>62</v>
+      </c>
       <c r="CZ93" s="29"/>
       <c r="DA93" s="29"/>
       <c r="DB93" s="29"/>
+      <c r="DC93" s="29"/>
     </row>
     <row r="94" spans="1:175" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="CY94" s="29"/>
       <c r="CZ94" s="29"/>
       <c r="DA94" s="29"/>
       <c r="DB94" s="29"/>
+      <c r="DC94" s="29"/>
     </row>
     <row r="95" spans="1:175" x14ac:dyDescent="0.2">
-      <c r="CY95" s="29"/>
       <c r="CZ95" s="29"/>
       <c r="DA95" s="29"/>
       <c r="DB95" s="29"/>
+      <c r="DC95" s="29"/>
     </row>
     <row r="96" spans="1:175" x14ac:dyDescent="0.2">
       <c r="A96" s="3"/>
@@ -20173,12 +20271,13 @@
       <c r="CV96" s="23"/>
       <c r="CW96" s="23"/>
       <c r="CX96" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="CY96" s="30"/>
+        <v>61</v>
+      </c>
+      <c r="CY96" s="23"/>
       <c r="CZ96" s="30"/>
       <c r="DA96" s="30"/>
       <c r="DB96" s="30"/>
+      <c r="DC96" s="30"/>
     </row>
     <row r="97" spans="1:175" x14ac:dyDescent="0.2">
       <c r="A97" s="4" t="s">
@@ -20487,17 +20586,20 @@
       <c r="CX97" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="CY97" s="31"/>
+      <c r="CY97" s="24" t="s">
+        <v>3</v>
+      </c>
       <c r="CZ97" s="31"/>
       <c r="DA97" s="31"/>
       <c r="DB97" s="31"/>
+      <c r="DC97" s="31"/>
     </row>
     <row r="98" spans="1:175" ht="10.9" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="6"/>
-      <c r="CY98" s="29"/>
       <c r="CZ98" s="29"/>
       <c r="DA98" s="29"/>
       <c r="DB98" s="29"/>
+      <c r="DC98" s="29"/>
     </row>
     <row r="99" spans="1:175" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
@@ -20804,13 +20906,15 @@
         <v>3.7927321752196548</v>
       </c>
       <c r="CX99" s="32">
-        <v>0.28772588745691507</v>
-      </c>
-      <c r="CY99" s="33"/>
+        <v>0.41339568712741936</v>
+      </c>
+      <c r="CY99" s="32">
+        <v>2.4303226745777238</v>
+      </c>
       <c r="CZ99" s="33"/>
       <c r="DA99" s="33"/>
       <c r="DB99" s="33"/>
-      <c r="DC99" s="8"/>
+      <c r="DC99" s="33"/>
       <c r="DD99" s="8"/>
       <c r="DE99" s="8"/>
       <c r="DF99" s="8"/>
@@ -21185,13 +21289,15 @@
         <v>-6.1365886567613046</v>
       </c>
       <c r="CX100" s="32">
-        <v>3.0541712181860277</v>
-      </c>
-      <c r="CY100" s="33"/>
+        <v>3.1157490082134558</v>
+      </c>
+      <c r="CY100" s="32">
+        <v>-1.8543638726639813</v>
+      </c>
       <c r="CZ100" s="33"/>
       <c r="DA100" s="33"/>
       <c r="DB100" s="33"/>
-      <c r="DC100" s="8"/>
+      <c r="DC100" s="33"/>
       <c r="DD100" s="8"/>
       <c r="DE100" s="8"/>
       <c r="DF100" s="8"/>
@@ -21566,13 +21672,15 @@
         <v>-1.0533477687317543</v>
       </c>
       <c r="CX101" s="32">
-        <v>12.25860284969977</v>
-      </c>
-      <c r="CY101" s="33"/>
+        <v>11.74620988324105</v>
+      </c>
+      <c r="CY101" s="32">
+        <v>7.8692708056122882</v>
+      </c>
       <c r="CZ101" s="33"/>
       <c r="DA101" s="33"/>
       <c r="DB101" s="33"/>
-      <c r="DC101" s="8"/>
+      <c r="DC101" s="33"/>
       <c r="DD101" s="8"/>
       <c r="DE101" s="8"/>
       <c r="DF101" s="8"/>
@@ -21947,13 +22055,15 @@
         <v>0.11345086296911688</v>
       </c>
       <c r="CX102" s="32">
-        <v>2.7208224282392734</v>
-      </c>
-      <c r="CY102" s="33"/>
+        <v>2.6058843573739381</v>
+      </c>
+      <c r="CY102" s="32">
+        <v>3.2240855196623528</v>
+      </c>
       <c r="CZ102" s="33"/>
       <c r="DA102" s="33"/>
       <c r="DB102" s="33"/>
-      <c r="DC102" s="8"/>
+      <c r="DC102" s="33"/>
       <c r="DD102" s="8"/>
       <c r="DE102" s="8"/>
       <c r="DF102" s="8"/>
@@ -22328,13 +22438,15 @@
         <v>-1.9626811850934303</v>
       </c>
       <c r="CX103" s="32">
-        <v>3.0911224344107495</v>
-      </c>
-      <c r="CY103" s="33"/>
+        <v>3.4837717894702536</v>
+      </c>
+      <c r="CY103" s="32">
+        <v>3.9445021790459833</v>
+      </c>
       <c r="CZ103" s="33"/>
       <c r="DA103" s="33"/>
       <c r="DB103" s="33"/>
-      <c r="DC103" s="8"/>
+      <c r="DC103" s="33"/>
       <c r="DD103" s="8"/>
       <c r="DE103" s="8"/>
       <c r="DF103" s="8"/>
@@ -22709,13 +22821,15 @@
         <v>5.6483077399349497</v>
       </c>
       <c r="CX104" s="32">
-        <v>5.6947308716537322</v>
-      </c>
-      <c r="CY104" s="33"/>
+        <v>5.9958657115663385</v>
+      </c>
+      <c r="CY104" s="32">
+        <v>9.7564513196541753</v>
+      </c>
       <c r="CZ104" s="33"/>
       <c r="DA104" s="33"/>
       <c r="DB104" s="33"/>
-      <c r="DC104" s="8"/>
+      <c r="DC104" s="33"/>
       <c r="DD104" s="8"/>
       <c r="DE104" s="8"/>
       <c r="DF104" s="8"/>
@@ -23090,13 +23204,15 @@
         <v>6.0058621655516049</v>
       </c>
       <c r="CX105" s="32">
-        <v>3.5374974360975955</v>
-      </c>
-      <c r="CY105" s="33"/>
+        <v>3.2622175692425657</v>
+      </c>
+      <c r="CY105" s="32">
+        <v>-7.490095902398437</v>
+      </c>
       <c r="CZ105" s="33"/>
       <c r="DA105" s="33"/>
       <c r="DB105" s="33"/>
-      <c r="DC105" s="8"/>
+      <c r="DC105" s="33"/>
       <c r="DD105" s="8"/>
       <c r="DE105" s="8"/>
       <c r="DF105" s="8"/>
@@ -23471,13 +23587,15 @@
         <v>3.5428482945700779</v>
       </c>
       <c r="CX106" s="32">
-        <v>5.6788768945325927</v>
-      </c>
-      <c r="CY106" s="33"/>
+        <v>5.5271154089896299</v>
+      </c>
+      <c r="CY106" s="32">
+        <v>5.5274421899457451</v>
+      </c>
       <c r="CZ106" s="33"/>
       <c r="DA106" s="33"/>
       <c r="DB106" s="33"/>
-      <c r="DC106" s="8"/>
+      <c r="DC106" s="33"/>
       <c r="DD106" s="8"/>
       <c r="DE106" s="8"/>
       <c r="DF106" s="8"/>
@@ -23852,13 +23970,15 @@
         <v>6.9813940197132212</v>
       </c>
       <c r="CX107" s="32">
-        <v>5.4334607994919395</v>
-      </c>
-      <c r="CY107" s="33"/>
+        <v>5.514794526284561</v>
+      </c>
+      <c r="CY107" s="32">
+        <v>-0.80896298538239364</v>
+      </c>
       <c r="CZ107" s="33"/>
       <c r="DA107" s="33"/>
       <c r="DB107" s="33"/>
-      <c r="DC107" s="8"/>
+      <c r="DC107" s="33"/>
       <c r="DD107" s="8"/>
       <c r="DE107" s="8"/>
       <c r="DF107" s="8"/>
@@ -24233,13 +24353,15 @@
         <v>6.6324016893898374</v>
       </c>
       <c r="CX108" s="32">
-        <v>6.7004239138229451</v>
-      </c>
-      <c r="CY108" s="33"/>
+        <v>6.4330277221809098</v>
+      </c>
+      <c r="CY108" s="32">
+        <v>12.957059293624411</v>
+      </c>
       <c r="CZ108" s="33"/>
       <c r="DA108" s="33"/>
       <c r="DB108" s="33"/>
-      <c r="DC108" s="8"/>
+      <c r="DC108" s="33"/>
       <c r="DD108" s="8"/>
       <c r="DE108" s="8"/>
       <c r="DF108" s="8"/>
@@ -24614,13 +24736,15 @@
         <v>7.0804187336179751</v>
       </c>
       <c r="CX109" s="32">
-        <v>4.2472837968456076</v>
-      </c>
-      <c r="CY109" s="33"/>
+        <v>4.5053321614979325</v>
+      </c>
+      <c r="CY109" s="32">
+        <v>-0.17575008673574644</v>
+      </c>
       <c r="CZ109" s="33"/>
       <c r="DA109" s="33"/>
       <c r="DB109" s="33"/>
-      <c r="DC109" s="8"/>
+      <c r="DC109" s="33"/>
       <c r="DD109" s="8"/>
       <c r="DE109" s="8"/>
       <c r="DF109" s="8"/>
@@ -24995,13 +25119,15 @@
         <v>3.9744610163546525</v>
       </c>
       <c r="CX110" s="32">
-        <v>4.0446280596069926</v>
-      </c>
-      <c r="CY110" s="33"/>
+        <v>3.9569188748360489</v>
+      </c>
+      <c r="CY110" s="32">
+        <v>5.7629819871159782</v>
+      </c>
       <c r="CZ110" s="33"/>
       <c r="DA110" s="33"/>
       <c r="DB110" s="33"/>
-      <c r="DC110" s="8"/>
+      <c r="DC110" s="33"/>
       <c r="DD110" s="8"/>
       <c r="DE110" s="8"/>
       <c r="DF110" s="8"/>
@@ -25173,11 +25299,11 @@
       <c r="CV111" s="26"/>
       <c r="CW111" s="26"/>
       <c r="CX111" s="26"/>
-      <c r="CY111" s="34"/>
+      <c r="CY111" s="26"/>
       <c r="CZ111" s="34"/>
       <c r="DA111" s="34"/>
       <c r="DB111" s="34"/>
-      <c r="DC111" s="8"/>
+      <c r="DC111" s="34"/>
       <c r="DD111" s="8"/>
       <c r="DE111" s="8"/>
       <c r="DF111" s="8"/>
@@ -25552,13 +25678,15 @@
         <v>3.7778645631406675</v>
       </c>
       <c r="CX112" s="32">
-        <v>3.0158187478206173</v>
-      </c>
-      <c r="CY112" s="33"/>
+        <v>3.0280184457533608</v>
+      </c>
+      <c r="CY112" s="32">
+        <v>2.8319698099088129</v>
+      </c>
       <c r="CZ112" s="33"/>
       <c r="DA112" s="33"/>
       <c r="DB112" s="33"/>
-      <c r="DC112" s="8"/>
+      <c r="DC112" s="33"/>
       <c r="DD112" s="8"/>
       <c r="DE112" s="8"/>
       <c r="DF112" s="8"/>
@@ -25731,19 +25859,20 @@
       <c r="CV113" s="27"/>
       <c r="CW113" s="27"/>
       <c r="CX113" s="27"/>
-      <c r="CY113" s="31"/>
+      <c r="CY113" s="27"/>
       <c r="CZ113" s="31"/>
       <c r="DA113" s="31"/>
       <c r="DB113" s="31"/>
+      <c r="DC113" s="31"/>
     </row>
     <row r="114" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A114" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="CY114" s="29"/>
       <c r="CZ114" s="29"/>
       <c r="DA114" s="29"/>
       <c r="DB114" s="29"/>
+      <c r="DC114" s="29"/>
     </row>
     <row r="115" spans="1:179" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B115" s="8"/>
@@ -25851,7 +25980,7 @@
       <c r="CZ115" s="35"/>
       <c r="DA115" s="35"/>
       <c r="DB115" s="26"/>
-      <c r="DC115" s="8"/>
+      <c r="DC115" s="26"/>
       <c r="DD115" s="8"/>
       <c r="DE115" s="8"/>
       <c r="DF115" s="8"/>
@@ -26027,7 +26156,7 @@
       <c r="CZ116" s="35"/>
       <c r="DA116" s="35"/>
       <c r="DB116" s="26"/>
-      <c r="DC116" s="8"/>
+      <c r="DC116" s="26"/>
       <c r="DD116" s="8"/>
       <c r="DE116" s="8"/>
       <c r="DF116" s="8"/>
@@ -26104,7 +26233,7 @@
     </row>
     <row r="118" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A118" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="120" spans="1:179" x14ac:dyDescent="0.2">
@@ -26114,7 +26243,7 @@
     </row>
     <row r="121" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A121" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="122" spans="1:179" x14ac:dyDescent="0.2">
@@ -26283,6 +26412,7 @@
       <c r="DB124" s="23">
         <v>2026</v>
       </c>
+      <c r="DC124" s="23"/>
     </row>
     <row r="125" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A125" s="4" t="s">
@@ -26602,6 +26732,9 @@
       </c>
       <c r="DB125" s="24" t="s">
         <v>2</v>
+      </c>
+      <c r="DC125" s="24" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="126" spans="1:179" ht="10.9" customHeight="1" x14ac:dyDescent="0.2">
@@ -26926,7 +27059,9 @@
       <c r="DB127" s="32">
         <v>133.11486788395311</v>
       </c>
-      <c r="DC127" s="8"/>
+      <c r="DC127" s="32">
+        <v>139.5972850202061</v>
+      </c>
       <c r="DD127" s="8"/>
       <c r="DE127" s="8"/>
       <c r="DF127" s="8"/>
@@ -27319,7 +27454,9 @@
       <c r="DB128" s="32">
         <v>179.82769105344306</v>
       </c>
-      <c r="DC128" s="8"/>
+      <c r="DC128" s="32">
+        <v>198.96518710056446</v>
+      </c>
       <c r="DD128" s="8"/>
       <c r="DE128" s="8"/>
       <c r="DF128" s="8"/>
@@ -27712,7 +27849,9 @@
       <c r="DB129" s="32">
         <v>120.13131886305874</v>
       </c>
-      <c r="DC129" s="8"/>
+      <c r="DC129" s="32">
+        <v>131.92034314191818</v>
+      </c>
       <c r="DD129" s="8"/>
       <c r="DE129" s="8"/>
       <c r="DF129" s="8"/>
@@ -28105,7 +28244,9 @@
       <c r="DB130" s="32">
         <v>120.18253008179754</v>
       </c>
-      <c r="DC130" s="8"/>
+      <c r="DC130" s="32">
+        <v>130.65607510578528</v>
+      </c>
       <c r="DD130" s="8"/>
       <c r="DE130" s="8"/>
       <c r="DF130" s="8"/>
@@ -28498,7 +28639,9 @@
       <c r="DB131" s="32">
         <v>128.86312316991368</v>
       </c>
-      <c r="DC131" s="8"/>
+      <c r="DC131" s="32">
+        <v>129.57998189279871</v>
+      </c>
       <c r="DD131" s="8"/>
       <c r="DE131" s="8"/>
       <c r="DF131" s="8"/>
@@ -28891,7 +29034,9 @@
       <c r="DB132" s="32">
         <v>122.77660735459482</v>
       </c>
-      <c r="DC132" s="8"/>
+      <c r="DC132" s="32">
+        <v>124.76083295503024</v>
+      </c>
       <c r="DD132" s="8"/>
       <c r="DE132" s="8"/>
       <c r="DF132" s="8"/>
@@ -29284,7 +29429,9 @@
       <c r="DB133" s="32">
         <v>137.80396639177681</v>
       </c>
-      <c r="DC133" s="8"/>
+      <c r="DC133" s="32">
+        <v>146.62817973403767</v>
+      </c>
       <c r="DD133" s="8"/>
       <c r="DE133" s="8"/>
       <c r="DF133" s="8"/>
@@ -29677,7 +29824,9 @@
       <c r="DB134" s="32">
         <v>107.18399324950228</v>
       </c>
-      <c r="DC134" s="8"/>
+      <c r="DC134" s="32">
+        <v>104.57676040538495</v>
+      </c>
       <c r="DD134" s="8"/>
       <c r="DE134" s="8"/>
       <c r="DF134" s="8"/>
@@ -30070,7 +30219,9 @@
       <c r="DB135" s="32">
         <v>120.35498636349908</v>
       </c>
-      <c r="DC135" s="8"/>
+      <c r="DC135" s="32">
+        <v>120.31810970100733</v>
+      </c>
       <c r="DD135" s="8"/>
       <c r="DE135" s="8"/>
       <c r="DF135" s="8"/>
@@ -30463,7 +30614,9 @@
       <c r="DB136" s="32">
         <v>120.37896764805924</v>
       </c>
-      <c r="DC136" s="8"/>
+      <c r="DC136" s="32">
+        <v>123.81360627057323</v>
+      </c>
       <c r="DD136" s="8"/>
       <c r="DE136" s="8"/>
       <c r="DF136" s="8"/>
@@ -30856,7 +31009,9 @@
       <c r="DB137" s="32">
         <v>135.83333333333334</v>
       </c>
-      <c r="DC137" s="8"/>
+      <c r="DC137" s="32">
+        <v>134.69803681330998</v>
+      </c>
       <c r="DD137" s="8"/>
       <c r="DE137" s="8"/>
       <c r="DF137" s="8"/>
@@ -31249,7 +31404,9 @@
       <c r="DB138" s="32">
         <v>131.73625706296522</v>
       </c>
-      <c r="DC138" s="8"/>
+      <c r="DC138" s="32">
+        <v>134.92874587520117</v>
+      </c>
       <c r="DD138" s="8"/>
       <c r="DE138" s="8"/>
       <c r="DF138" s="8"/>
@@ -31429,7 +31586,7 @@
       <c r="CZ139" s="26"/>
       <c r="DA139" s="26"/>
       <c r="DB139" s="26"/>
-      <c r="DC139" s="8"/>
+      <c r="DC139" s="26"/>
       <c r="DD139" s="8"/>
       <c r="DE139" s="8"/>
       <c r="DF139" s="8"/>
@@ -31820,9 +31977,11 @@
         <v>125.75245526872317</v>
       </c>
       <c r="DB140" s="32">
-        <v>130.06285010024203</v>
-      </c>
-      <c r="DC140" s="8"/>
+        <v>130.06688920311512</v>
+      </c>
+      <c r="DC140" s="32">
+        <v>135.07714627918344</v>
+      </c>
       <c r="DD140" s="8"/>
       <c r="DE140" s="8"/>
       <c r="DF140" s="8"/>
@@ -32003,6 +32162,7 @@
       <c r="CZ141" s="27"/>
       <c r="DA141" s="27"/>
       <c r="DB141" s="27"/>
+      <c r="DC141" s="27"/>
     </row>
     <row r="142" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A142" s="12" t="s">
@@ -32021,7 +32181,7 @@
     </row>
     <row r="147" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A147" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="149" spans="1:179" x14ac:dyDescent="0.2">
@@ -32031,7 +32191,7 @@
     </row>
     <row r="150" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A150" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="151" spans="1:179" x14ac:dyDescent="0.2">
@@ -32200,6 +32360,7 @@
       <c r="DB153" s="23">
         <v>2026</v>
       </c>
+      <c r="DC153" s="23"/>
     </row>
     <row r="154" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A154" s="4" t="s">
@@ -32519,6 +32680,9 @@
       </c>
       <c r="DB154" s="24" t="s">
         <v>2</v>
+      </c>
+      <c r="DC154" s="24" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="155" spans="1:179" ht="10.9" customHeight="1" x14ac:dyDescent="0.2">
@@ -32841,9 +33005,11 @@
         <v>37.35495101165894</v>
       </c>
       <c r="DB156" s="32">
-        <v>32.617855510780672</v>
-      </c>
-      <c r="DC156" s="8"/>
+        <v>32.653847468507472</v>
+      </c>
+      <c r="DC156" s="32">
+        <v>37.510123201983355</v>
+      </c>
       <c r="DD156" s="8"/>
       <c r="DE156" s="8"/>
       <c r="DF156" s="8"/>
@@ -33234,9 +33400,11 @@
         <v>1.9897456335966761</v>
       </c>
       <c r="DB157" s="32">
-        <v>1.8035476286195591</v>
-      </c>
-      <c r="DC157" s="8"/>
+        <v>1.8043555768871784</v>
+      </c>
+      <c r="DC157" s="32">
+        <v>1.6143908878409261</v>
+      </c>
       <c r="DD157" s="8"/>
       <c r="DE157" s="8"/>
       <c r="DF157" s="8"/>
@@ -33627,9 +33795,11 @@
         <v>1.5676254952267776</v>
       </c>
       <c r="DB158" s="32">
-        <v>1.3754731629479835</v>
-      </c>
-      <c r="DC158" s="8"/>
+        <v>1.3689903133212518</v>
+      </c>
+      <c r="DC158" s="32">
+        <v>1.0564912401759921</v>
+      </c>
       <c r="DD158" s="8"/>
       <c r="DE158" s="8"/>
       <c r="DF158" s="8"/>
@@ -34020,9 +34190,11 @@
         <v>10.450112164051506</v>
       </c>
       <c r="DB159" s="32">
-        <v>10.959719702513523</v>
-      </c>
-      <c r="DC159" s="8"/>
+        <v>10.945820245993893</v>
+      </c>
+      <c r="DC159" s="32">
+        <v>14.510308867216617</v>
+      </c>
       <c r="DD159" s="8"/>
       <c r="DE159" s="8"/>
       <c r="DF159" s="8"/>
@@ -34413,9 +34585,11 @@
         <v>2.4403664072674704</v>
       </c>
       <c r="DB160" s="32">
-        <v>2.3748278876814086</v>
-      </c>
-      <c r="DC160" s="8"/>
+        <v>2.3835167393984507</v>
+      </c>
+      <c r="DC160" s="32">
+        <v>2.3626123586021253</v>
+      </c>
       <c r="DD160" s="8"/>
       <c r="DE160" s="8"/>
       <c r="DF160" s="8"/>
@@ -34806,9 +34980,11 @@
         <v>4.4588421426957927</v>
       </c>
       <c r="DB161" s="32">
-        <v>4.5933686278660755</v>
-      </c>
-      <c r="DC161" s="8"/>
+        <v>4.6057671043890256</v>
+      </c>
+      <c r="DC161" s="32">
+        <v>4.1341507063178611</v>
+      </c>
       <c r="DD161" s="8"/>
       <c r="DE161" s="8"/>
       <c r="DF161" s="8"/>
@@ -35199,9 +35375,11 @@
         <v>8.2180309363383532</v>
       </c>
       <c r="DB162" s="32">
-        <v>10.920402074268493</v>
-      </c>
-      <c r="DC162" s="8"/>
+        <v>10.889739659520545</v>
+      </c>
+      <c r="DC162" s="32">
+        <v>9.5207362281610344</v>
+      </c>
       <c r="DD162" s="8"/>
       <c r="DE162" s="8"/>
       <c r="DF162" s="8"/>
@@ -35592,9 +35770,11 @@
         <v>2.4102637552467896</v>
       </c>
       <c r="DB163" s="32">
-        <v>2.7824009136202443</v>
-      </c>
-      <c r="DC163" s="8"/>
+        <v>2.7779899461416542</v>
+      </c>
+      <c r="DC163" s="32">
+        <v>2.9260634623734672</v>
+      </c>
       <c r="DD163" s="8"/>
       <c r="DE163" s="8"/>
       <c r="DF163" s="8"/>
@@ -35985,9 +36165,11 @@
         <v>1.9207835906935355</v>
       </c>
       <c r="DB164" s="32">
-        <v>1.917862352745934</v>
-      </c>
-      <c r="DC164" s="8"/>
+        <v>1.9190549662716081</v>
+      </c>
+      <c r="DC164" s="32">
+        <v>1.3008216186818018</v>
+      </c>
       <c r="DD164" s="8"/>
       <c r="DE164" s="8"/>
       <c r="DF164" s="8"/>
@@ -36378,9 +36560,11 @@
         <v>4.9640629602150677</v>
       </c>
       <c r="DB165" s="32">
-        <v>5.5261147905211487</v>
-      </c>
-      <c r="DC165" s="8"/>
+        <v>5.511442218211517</v>
+      </c>
+      <c r="DC165" s="32">
+        <v>5.2710666373929707</v>
+      </c>
       <c r="DD165" s="8"/>
       <c r="DE165" s="8"/>
       <c r="DF165" s="8"/>
@@ -36771,9 +36955,11 @@
         <v>9.1027974592063732</v>
       </c>
       <c r="DB166" s="32">
-        <v>10.845627002812328</v>
-      </c>
-      <c r="DC166" s="8"/>
+        <v>10.870848690316857</v>
+      </c>
+      <c r="DC166" s="32">
+        <v>6.0475701259431496</v>
+      </c>
       <c r="DD166" s="8"/>
       <c r="DE166" s="8"/>
       <c r="DF166" s="8"/>
@@ -37164,9 +37350,11 @@
         <v>15.122418443802719</v>
       </c>
       <c r="DB167" s="32">
-        <v>14.282800345622624</v>
-      </c>
-      <c r="DC167" s="8"/>
+        <v>14.268627071040557</v>
+      </c>
+      <c r="DC167" s="32">
+        <v>13.745664665310715</v>
+      </c>
       <c r="DD167" s="8"/>
       <c r="DE167" s="8"/>
       <c r="DF167" s="8"/>
@@ -37346,7 +37534,7 @@
       <c r="CZ168" s="26"/>
       <c r="DA168" s="26"/>
       <c r="DB168" s="26"/>
-      <c r="DC168" s="8"/>
+      <c r="DC168" s="26"/>
       <c r="DD168" s="8"/>
       <c r="DE168" s="8"/>
       <c r="DF168" s="8"/>
@@ -37739,7 +37927,9 @@
       <c r="DB169" s="32">
         <v>100</v>
       </c>
-      <c r="DC169" s="8"/>
+      <c r="DC169" s="32">
+        <v>100</v>
+      </c>
       <c r="DD169" s="8"/>
       <c r="DE169" s="8"/>
       <c r="DF169" s="8"/>
@@ -37920,6 +38110,7 @@
       <c r="CZ170" s="27"/>
       <c r="DA170" s="27"/>
       <c r="DB170" s="27"/>
+      <c r="DC170" s="27"/>
     </row>
     <row r="171" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A171" s="12" t="s">
@@ -38032,7 +38223,7 @@
       <c r="CZ172" s="26"/>
       <c r="DA172" s="26"/>
       <c r="DB172" s="26"/>
-      <c r="DC172" s="8"/>
+      <c r="DC172" s="26"/>
       <c r="DD172" s="8"/>
       <c r="DE172" s="8"/>
       <c r="DF172" s="8"/>
@@ -38212,7 +38403,7 @@
       <c r="CZ173" s="26"/>
       <c r="DA173" s="26"/>
       <c r="DB173" s="26"/>
-      <c r="DC173" s="8"/>
+      <c r="DC173" s="26"/>
       <c r="DD173" s="8"/>
       <c r="DE173" s="8"/>
       <c r="DF173" s="8"/>
@@ -38298,7 +38489,7 @@
     </row>
     <row r="176" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A176" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="178" spans="1:179" x14ac:dyDescent="0.2">
@@ -38308,7 +38499,7 @@
     </row>
     <row r="179" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A179" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="180" spans="1:179" x14ac:dyDescent="0.2">
@@ -38477,6 +38668,7 @@
       <c r="DB182" s="23">
         <v>2026</v>
       </c>
+      <c r="DC182" s="23"/>
     </row>
     <row r="183" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A183" s="4" t="s">
@@ -38796,6 +38988,9 @@
       </c>
       <c r="DB183" s="24" t="s">
         <v>2</v>
+      </c>
+      <c r="DC183" s="24" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="184" spans="1:179" ht="10.9" customHeight="1" x14ac:dyDescent="0.2">
@@ -39118,9 +39313,11 @@
         <v>35.622626491414316</v>
       </c>
       <c r="DB185" s="32">
-        <v>31.870003098289786</v>
-      </c>
-      <c r="DC185" s="8"/>
+        <v>31.906160658510313</v>
+      </c>
+      <c r="DC185" s="32">
+        <v>36.295551148943247</v>
+      </c>
       <c r="DD185" s="8"/>
       <c r="DE185" s="8"/>
       <c r="DF185" s="8"/>
@@ -39511,9 +39708,11 @@
         <v>1.3928558482030335</v>
       </c>
       <c r="DB186" s="32">
-        <v>1.3044406203273744</v>
-      </c>
-      <c r="DC186" s="8"/>
+        <v>1.3050655075822601</v>
+      </c>
+      <c r="DC186" s="32">
+        <v>1.0960073834346216</v>
+      </c>
       <c r="DD186" s="8"/>
       <c r="DE186" s="8"/>
       <c r="DF186" s="8"/>
@@ -39904,9 +40103,11 @@
         <v>1.6739075855519421</v>
       </c>
       <c r="DB187" s="32">
-        <v>1.4891866792317539</v>
-      </c>
-      <c r="DC187" s="8"/>
+        <v>1.4822139063158819</v>
+      </c>
+      <c r="DC187" s="32">
+        <v>1.0817726697269516</v>
+      </c>
       <c r="DD187" s="8"/>
       <c r="DE187" s="8"/>
       <c r="DF187" s="8"/>
@@ -40297,9 +40498,11 @@
         <v>10.440580907306169</v>
       </c>
       <c r="DB188" s="32">
-        <v>11.860728675278406</v>
-      </c>
-      <c r="DC188" s="8"/>
+        <v>11.846054399120439</v>
+      </c>
+      <c r="DC188" s="32">
+        <v>15.001301025047894</v>
+      </c>
       <c r="DD188" s="8"/>
       <c r="DE188" s="8"/>
       <c r="DF188" s="8"/>
@@ -40690,9 +40893,11 @@
         <v>2.4991936999721429</v>
       </c>
       <c r="DB189" s="32">
-        <v>2.3969377427094405</v>
-      </c>
-      <c r="DC189" s="8"/>
+        <v>2.405782197660483</v>
+      </c>
+      <c r="DC189" s="32">
+        <v>2.462841331679809</v>
+      </c>
       <c r="DD189" s="8"/>
       <c r="DE189" s="8"/>
       <c r="DF189" s="8"/>
@@ -41083,9 +41288,11 @@
         <v>4.4857597563020342</v>
       </c>
       <c r="DB190" s="32">
-        <v>4.865964520227001</v>
-      </c>
-      <c r="DC190" s="8"/>
+        <v>4.8792503113542063</v>
+      </c>
+      <c r="DC190" s="32">
+        <v>4.4759983279269377</v>
+      </c>
       <c r="DD190" s="8"/>
       <c r="DE190" s="8"/>
       <c r="DF190" s="8"/>
@@ -41476,9 +41683,11 @@
         <v>8.1432744910178165</v>
       </c>
       <c r="DB191" s="32">
-        <v>10.306950193160123</v>
-      </c>
-      <c r="DC191" s="8"/>
+        <v>10.278329418464024</v>
+      </c>
+      <c r="DC191" s="32">
+        <v>8.7707143504714367</v>
+      </c>
       <c r="DD191" s="8"/>
       <c r="DE191" s="8"/>
       <c r="DF191" s="8"/>
@@ -41869,9 +42078,11 @@
         <v>3.0543196119418572</v>
       </c>
       <c r="DB192" s="32">
-        <v>3.3763156416888469</v>
-      </c>
-      <c r="DC192" s="8"/>
+        <v>3.3710678206500968</v>
+      </c>
+      <c r="DC192" s="32">
+        <v>3.7794659233758652</v>
+      </c>
       <c r="DD192" s="8"/>
       <c r="DE192" s="8"/>
       <c r="DF192" s="8"/>
@@ -42262,9 +42473,11 @@
         <v>2.0556348418543737</v>
       </c>
       <c r="DB193" s="32">
-        <v>2.0725576167215798</v>
-      </c>
-      <c r="DC193" s="8"/>
+        <v>2.073910830074563</v>
+      </c>
+      <c r="DC193" s="32">
+        <v>1.4603892340600397</v>
+      </c>
       <c r="DD193" s="8"/>
       <c r="DE193" s="8"/>
       <c r="DF193" s="8"/>
@@ -42655,9 +42868,11 @@
         <v>5.4668335274871662</v>
       </c>
       <c r="DB194" s="32">
-        <v>5.9706629295709055</v>
-      </c>
-      <c r="DC194" s="8"/>
+        <v>5.95499494929458</v>
+      </c>
+      <c r="DC194" s="32">
+        <v>5.7505847755577006</v>
+      </c>
       <c r="DD194" s="8"/>
       <c r="DE194" s="8"/>
       <c r="DF194" s="8"/>
@@ -43048,9 +43263,11 @@
         <v>8.7430583183304122</v>
       </c>
       <c r="DB195" s="32">
-        <v>10.384882152956447</v>
-      </c>
-      <c r="DC195" s="8"/>
+        <v>10.409355623170098</v>
+      </c>
+      <c r="DC195" s="32">
+        <v>6.0645910947302175</v>
+      </c>
       <c r="DD195" s="8"/>
       <c r="DE195" s="8"/>
       <c r="DF195" s="8"/>
@@ -43441,9 +43658,11 @@
         <v>16.421954920618724</v>
       </c>
       <c r="DB196" s="32">
-        <v>14.101370129838322</v>
-      </c>
-      <c r="DC196" s="8"/>
+        <v>14.08781437780306</v>
+      </c>
+      <c r="DC196" s="32">
+        <v>13.760782735045263</v>
+      </c>
       <c r="DD196" s="8"/>
       <c r="DE196" s="8"/>
       <c r="DF196" s="8"/>
@@ -43623,7 +43842,7 @@
       <c r="CZ197" s="26"/>
       <c r="DA197" s="26"/>
       <c r="DB197" s="26"/>
-      <c r="DC197" s="8"/>
+      <c r="DC197" s="26"/>
       <c r="DD197" s="8"/>
       <c r="DE197" s="8"/>
       <c r="DF197" s="8"/>
@@ -44016,7 +44235,9 @@
       <c r="DB198" s="32">
         <v>100</v>
       </c>
-      <c r="DC198" s="8"/>
+      <c r="DC198" s="32">
+        <v>100</v>
+      </c>
       <c r="DD198" s="8"/>
       <c r="DE198" s="8"/>
       <c r="DF198" s="8"/>
@@ -44197,6 +44418,7 @@
       <c r="CZ199" s="27"/>
       <c r="DA199" s="27"/>
       <c r="DB199" s="27"/>
+      <c r="DC199" s="27"/>
     </row>
     <row r="200" spans="1:179" x14ac:dyDescent="0.2">
       <c r="A200" s="12" t="s">
@@ -44310,7 +44532,7 @@
       <c r="CZ201" s="36"/>
       <c r="DA201" s="36"/>
       <c r="DB201" s="36"/>
-      <c r="DC201" s="20"/>
+      <c r="DC201" s="36"/>
       <c r="DD201" s="20"/>
       <c r="DE201" s="20"/>
       <c r="DF201" s="20"/>
@@ -44385,25 +44607,30 @@
       <c r="FW201" s="20"/>
     </row>
     <row r="202" spans="1:179" x14ac:dyDescent="0.2">
-      <c r="CX202" s="29"/>
-      <c r="CY202" s="29"/>
-      <c r="CZ202" s="29"/>
-      <c r="DA202" s="29"/>
+      <c r="CX202" s="28"/>
+      <c r="CZ202" s="28"/>
+      <c r="DA202" s="28"/>
       <c r="DB202" s="28"/>
     </row>
     <row r="203" spans="1:179" x14ac:dyDescent="0.2">
       <c r="CT203" s="28"/>
       <c r="CV203" s="28"/>
       <c r="CX203" s="28"/>
+      <c r="CY203" s="28"/>
       <c r="CZ203" s="28"/>
       <c r="DA203" s="28"/>
+      <c r="DB203" s="28"/>
+      <c r="DC203" s="28"/>
     </row>
     <row r="204" spans="1:179" x14ac:dyDescent="0.2">
       <c r="CT204" s="28"/>
       <c r="CV204" s="28"/>
       <c r="CX204" s="28"/>
+      <c r="CY204" s="28"/>
       <c r="CZ204" s="28"/>
       <c r="DA204" s="28"/>
+      <c r="DB204" s="28"/>
+      <c r="DC204" s="28"/>
     </row>
     <row r="205" spans="1:179" x14ac:dyDescent="0.2">
       <c r="CT205" s="28"/>
@@ -44413,24 +44640,18 @@
       <c r="CY205" s="28"/>
       <c r="CZ205" s="28"/>
       <c r="DA205" s="28"/>
+      <c r="DB205" s="28"/>
+      <c r="DC205" s="28"/>
     </row>
     <row r="206" spans="1:179" x14ac:dyDescent="0.2">
       <c r="CT206" s="28"/>
       <c r="CU206" s="28"/>
       <c r="CV206" s="28"/>
-      <c r="CX206" s="28"/>
-      <c r="CY206" s="28"/>
-      <c r="CZ206" s="28"/>
-      <c r="DA206" s="28"/>
     </row>
     <row r="207" spans="1:179" x14ac:dyDescent="0.2">
       <c r="CT207" s="28"/>
       <c r="CU207" s="28"/>
       <c r="CV207" s="28"/>
-      <c r="CX207" s="28"/>
-      <c r="CY207" s="28"/>
-      <c r="CZ207" s="28"/>
-      <c r="DA207" s="28"/>
     </row>
   </sheetData>
   <pageMargins left="0.3" right="0.3" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>